<commit_message>
Updating files for 12/1
</commit_message>
<xml_diff>
--- a/data_raw/smelt/abundance_estimates.xlsx
+++ b/data_raw/smelt/abundance_estimates.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://doimspp-my.sharepoint.com/personal/cpien_usbr_gov/Documents/Work/GitHub/samt_smt_assessments/data_raw/smelt/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://doimspp-my.sharepoint.com/personal/lmccormick_usbr_gov/Documents/Documents/Research/R/samt_smt_assessments/data_raw/smelt/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="25" documentId="8_{BF3B047A-36C0-4AD4-A0BA-7FD3D60567F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{35FB7A12-4F86-463A-AE32-53D466ECC9BB}"/>
+  <xr:revisionPtr revIDLastSave="38" documentId="8_{BF3B047A-36C0-4AD4-A0BA-7FD3D60567F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5E334DD1-4CE3-4A54-9107-613145A2883D}"/>
   <bookViews>
-    <workbookView xWindow="-24240" yWindow="2415" windowWidth="21600" windowHeight="12645" xr2:uid="{03E7A685-4EE0-4A4E-B4B4-B1F660F8462C}"/>
+    <workbookView xWindow="1920" yWindow="1920" windowWidth="17280" windowHeight="8880" activeTab="1" xr2:uid="{03E7A685-4EE0-4A4E-B4B4-B1F660F8462C}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="644" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="696" uniqueCount="47">
   <si>
     <t>Week</t>
   </si>
@@ -173,6 +173,12 @@
   <si>
     <t>November 10–14, 2025</t>
   </si>
+  <si>
+    <t>November 17–21, 2025</t>
+  </si>
+  <si>
+    <t>November 24–28, 2025</t>
+  </si>
 </sst>
 </file>
 
@@ -225,6 +231,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -544,14 +554,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{91E6CDBE-81F8-437E-8236-059C4BBF9395}">
-  <dimension ref="A1:K164"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:K178"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="19.85546875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="16.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="19.88671875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="16.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -586,7 +596,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>1</v>
       </c>
@@ -621,7 +631,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>1</v>
       </c>
@@ -656,7 +666,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>1</v>
       </c>
@@ -691,7 +701,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>1</v>
       </c>
@@ -726,7 +736,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>1</v>
       </c>
@@ -761,7 +771,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>1</v>
       </c>
@@ -796,7 +806,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>1</v>
       </c>
@@ -831,7 +841,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>2</v>
       </c>
@@ -866,7 +876,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>2</v>
       </c>
@@ -901,7 +911,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>2</v>
       </c>
@@ -936,7 +946,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A12">
         <v>2</v>
       </c>
@@ -971,7 +981,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>2</v>
       </c>
@@ -1006,7 +1016,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A14">
         <v>2</v>
       </c>
@@ -1041,7 +1051,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A15">
         <v>2</v>
       </c>
@@ -1076,7 +1086,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A16">
         <v>3</v>
       </c>
@@ -1111,7 +1121,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A17">
         <v>3</v>
       </c>
@@ -1146,7 +1156,7 @@
         <v>3490</v>
       </c>
     </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A18">
         <v>3</v>
       </c>
@@ -1181,7 +1191,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A19">
         <v>3</v>
       </c>
@@ -1216,7 +1226,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A20">
         <v>3</v>
       </c>
@@ -1251,7 +1261,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A21">
         <v>3</v>
       </c>
@@ -1286,7 +1296,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A22">
         <v>3</v>
       </c>
@@ -1321,7 +1331,7 @@
         <v>3490</v>
       </c>
     </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A23">
         <v>4</v>
       </c>
@@ -1356,7 +1366,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A24">
         <v>4</v>
       </c>
@@ -1391,7 +1401,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A25">
         <v>4</v>
       </c>
@@ -1426,7 +1436,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A26">
         <v>4</v>
       </c>
@@ -1461,7 +1471,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A27">
         <v>4</v>
       </c>
@@ -1496,7 +1506,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A28">
         <v>4</v>
       </c>
@@ -1531,7 +1541,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="29" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A29">
         <v>4</v>
       </c>
@@ -1566,7 +1576,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="30" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A30">
         <v>5</v>
       </c>
@@ -1601,7 +1611,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="31" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A31">
         <v>5</v>
       </c>
@@ -1636,7 +1646,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="32" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A32">
         <v>5</v>
       </c>
@@ -1671,7 +1681,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="33" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A33">
         <v>5</v>
       </c>
@@ -1706,7 +1716,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="34" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A34">
         <v>5</v>
       </c>
@@ -1741,7 +1751,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="35" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A35">
         <v>5</v>
       </c>
@@ -1776,7 +1786,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="36" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A36">
         <v>5</v>
       </c>
@@ -1811,7 +1821,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="37" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A37">
         <v>6</v>
       </c>
@@ -1846,7 +1856,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="38" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A38">
         <v>6</v>
       </c>
@@ -1881,7 +1891,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="39" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A39">
         <v>6</v>
       </c>
@@ -1916,7 +1926,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="40" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A40">
         <v>6</v>
       </c>
@@ -1951,7 +1961,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="41" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A41">
         <v>6</v>
       </c>
@@ -1986,7 +1996,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="42" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A42">
         <v>6</v>
       </c>
@@ -2021,7 +2031,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="43" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A43">
         <v>6</v>
       </c>
@@ -2056,7 +2066,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="44" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A44">
         <v>7</v>
       </c>
@@ -2091,7 +2101,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="45" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A45">
         <v>7</v>
       </c>
@@ -2126,7 +2136,7 @@
         <v>3307</v>
       </c>
     </row>
-    <row r="46" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A46">
         <v>7</v>
       </c>
@@ -2161,7 +2171,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="47" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A47">
         <v>7</v>
       </c>
@@ -2196,7 +2206,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="48" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A48">
         <v>7</v>
       </c>
@@ -2231,7 +2241,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="49" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A49">
         <v>7</v>
       </c>
@@ -2266,7 +2276,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="50" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A50">
         <v>7</v>
       </c>
@@ -2301,7 +2311,7 @@
         <v>3307</v>
       </c>
     </row>
-    <row r="51" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A51">
         <v>8</v>
       </c>
@@ -2336,7 +2346,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="52" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A52">
         <v>8</v>
       </c>
@@ -2371,7 +2381,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="53" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A53">
         <v>8</v>
       </c>
@@ -2406,7 +2416,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="54" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A54">
         <v>8</v>
       </c>
@@ -2441,7 +2451,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="55" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A55">
         <v>8</v>
       </c>
@@ -2476,7 +2486,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="56" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A56">
         <v>8</v>
       </c>
@@ -2511,7 +2521,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="57" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A57">
         <v>8</v>
       </c>
@@ -2546,7 +2556,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="58" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A58">
         <v>9</v>
       </c>
@@ -2581,7 +2591,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="59" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A59">
         <v>9</v>
       </c>
@@ -2616,7 +2626,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="60" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A60">
         <v>9</v>
       </c>
@@ -2651,7 +2661,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="61" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A61">
         <v>9</v>
       </c>
@@ -2686,7 +2696,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="62" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A62">
         <v>9</v>
       </c>
@@ -2721,7 +2731,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="63" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A63">
         <v>9</v>
       </c>
@@ -2756,7 +2766,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="64" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A64">
         <v>9</v>
       </c>
@@ -2791,7 +2801,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="65" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A65">
         <v>10</v>
       </c>
@@ -2826,7 +2836,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="66" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A66">
         <v>10</v>
       </c>
@@ -2861,7 +2871,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="67" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A67">
         <v>10</v>
       </c>
@@ -2896,7 +2906,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="68" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A68">
         <v>10</v>
       </c>
@@ -2931,7 +2941,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="69" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A69">
         <v>10</v>
       </c>
@@ -2966,7 +2976,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="70" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A70">
         <v>10</v>
       </c>
@@ -3001,7 +3011,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="71" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A71">
         <v>10</v>
       </c>
@@ -3036,7 +3046,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="72" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A72">
         <v>11</v>
       </c>
@@ -3071,7 +3081,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="73" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A73">
         <v>11</v>
       </c>
@@ -3106,7 +3116,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="74" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A74">
         <v>11</v>
       </c>
@@ -3141,7 +3151,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="75" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A75">
         <v>11</v>
       </c>
@@ -3176,7 +3186,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="76" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A76">
         <v>11</v>
       </c>
@@ -3211,7 +3221,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="77" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A77">
         <v>11</v>
       </c>
@@ -3246,7 +3256,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="78" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A78">
         <v>11</v>
       </c>
@@ -3281,7 +3291,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="79" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A79">
         <v>12</v>
       </c>
@@ -3316,7 +3326,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="80" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A80">
         <v>12</v>
       </c>
@@ -3351,7 +3361,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="81" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A81">
         <v>12</v>
       </c>
@@ -3386,7 +3396,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="82" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A82">
         <v>12</v>
       </c>
@@ -3421,7 +3431,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="83" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A83">
         <v>12</v>
       </c>
@@ -3456,7 +3466,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="84" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A84">
         <v>12</v>
       </c>
@@ -3491,7 +3501,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="85" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A85">
         <v>12</v>
       </c>
@@ -3526,7 +3536,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="86" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A86">
         <v>13</v>
       </c>
@@ -3561,7 +3571,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="87" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A87">
         <v>13</v>
       </c>
@@ -3596,7 +3606,7 @@
         <v>3302</v>
       </c>
     </row>
-    <row r="88" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A88">
         <v>13</v>
       </c>
@@ -3631,7 +3641,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="89" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A89">
         <v>13</v>
       </c>
@@ -3666,7 +3676,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="90" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A90">
         <v>13</v>
       </c>
@@ -3701,7 +3711,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="91" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A91">
         <v>13</v>
       </c>
@@ -3736,7 +3746,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="92" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A92">
         <v>13</v>
       </c>
@@ -3771,7 +3781,7 @@
         <v>3302</v>
       </c>
     </row>
-    <row r="93" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A93">
         <v>14</v>
       </c>
@@ -3806,7 +3816,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="94" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A94">
         <v>14</v>
       </c>
@@ -3841,7 +3851,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="95" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A95">
         <v>14</v>
       </c>
@@ -3876,7 +3886,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="96" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A96">
         <v>14</v>
       </c>
@@ -3911,7 +3921,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="97" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A97">
         <v>14</v>
       </c>
@@ -3946,7 +3956,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="98" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A98">
         <v>14</v>
       </c>
@@ -3981,7 +3991,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="99" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A99">
         <v>14</v>
       </c>
@@ -4016,7 +4026,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="100" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A100">
         <v>15</v>
       </c>
@@ -4051,7 +4061,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="101" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A101">
         <v>15</v>
       </c>
@@ -4086,7 +4096,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="102" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A102">
         <v>16</v>
       </c>
@@ -4121,7 +4131,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="103" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A103">
         <v>16</v>
       </c>
@@ -4156,7 +4166,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="104" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A104">
         <v>16</v>
       </c>
@@ -4191,7 +4201,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="105" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A105">
         <v>16</v>
       </c>
@@ -4226,7 +4236,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="106" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A106">
         <v>16</v>
       </c>
@@ -4261,7 +4271,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="107" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A107">
         <v>16</v>
       </c>
@@ -4296,7 +4306,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="108" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A108">
         <v>16</v>
       </c>
@@ -4331,7 +4341,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="109" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A109">
         <v>17</v>
       </c>
@@ -4366,7 +4376,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="110" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A110">
         <v>17</v>
       </c>
@@ -4401,7 +4411,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="111" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A111">
         <v>17</v>
       </c>
@@ -4436,7 +4446,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="112" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A112">
         <v>17</v>
       </c>
@@ -4471,7 +4481,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="113" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A113">
         <v>17</v>
       </c>
@@ -4506,7 +4516,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="114" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A114">
         <v>17</v>
       </c>
@@ -4541,7 +4551,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="115" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A115">
         <v>17</v>
       </c>
@@ -4576,7 +4586,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="116" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A116">
         <v>18</v>
       </c>
@@ -4611,7 +4621,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="117" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A117">
         <v>18</v>
       </c>
@@ -4646,7 +4656,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="118" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A118">
         <v>18</v>
       </c>
@@ -4681,7 +4691,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="119" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A119">
         <v>18</v>
       </c>
@@ -4716,7 +4726,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="120" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A120">
         <v>18</v>
       </c>
@@ -4751,7 +4761,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="121" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A121">
         <v>18</v>
       </c>
@@ -4786,7 +4796,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="122" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A122">
         <v>18</v>
       </c>
@@ -4821,7 +4831,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="123" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A123">
         <v>19</v>
       </c>
@@ -4856,7 +4866,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="124" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A124">
         <v>19</v>
       </c>
@@ -4891,7 +4901,7 @@
         <v>3115</v>
       </c>
     </row>
-    <row r="125" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A125">
         <v>19</v>
       </c>
@@ -4926,7 +4936,7 @@
         <v>1596</v>
       </c>
     </row>
-    <row r="126" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A126">
         <v>19</v>
       </c>
@@ -4961,7 +4971,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="127" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A127">
         <v>19</v>
       </c>
@@ -4996,7 +5006,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="128" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A128">
         <v>19</v>
       </c>
@@ -5031,7 +5041,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="129" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A129">
         <v>19</v>
       </c>
@@ -5066,7 +5076,7 @@
         <v>3859</v>
       </c>
     </row>
-    <row r="130" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A130">
         <v>20</v>
       </c>
@@ -5101,7 +5111,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="131" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A131">
         <v>20</v>
       </c>
@@ -5136,7 +5146,7 @@
         <v>3336</v>
       </c>
     </row>
-    <row r="132" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A132">
         <v>20</v>
       </c>
@@ -5171,7 +5181,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="133" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A133">
         <v>20</v>
       </c>
@@ -5206,7 +5216,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="134" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A134">
         <v>20</v>
       </c>
@@ -5241,7 +5251,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="135" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A135">
         <v>20</v>
       </c>
@@ -5276,7 +5286,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="136" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A136">
         <v>20</v>
       </c>
@@ -5311,7 +5321,7 @@
         <v>3336</v>
       </c>
     </row>
-    <row r="137" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A137">
         <v>21</v>
       </c>
@@ -5346,7 +5356,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="138" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A138">
         <v>21</v>
       </c>
@@ -5381,7 +5391,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="139" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A139">
         <v>21</v>
       </c>
@@ -5416,7 +5426,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="140" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A140">
         <v>21</v>
       </c>
@@ -5451,7 +5461,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="141" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A141">
         <v>21</v>
       </c>
@@ -5486,7 +5496,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="142" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A142">
         <v>21</v>
       </c>
@@ -5521,7 +5531,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="143" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A143">
         <v>21</v>
       </c>
@@ -5556,7 +5566,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="144" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A144">
         <v>22</v>
       </c>
@@ -5591,7 +5601,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="145" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A145">
         <v>22</v>
       </c>
@@ -5626,7 +5636,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="146" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="146" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A146">
         <v>22</v>
       </c>
@@ -5661,7 +5671,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="147" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A147">
         <v>22</v>
       </c>
@@ -5696,7 +5706,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="148" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A148">
         <v>22</v>
       </c>
@@ -5731,7 +5741,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="149" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A149">
         <v>22</v>
       </c>
@@ -5766,7 +5776,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="150" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A150">
         <v>22</v>
       </c>
@@ -5801,7 +5811,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="151" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="151" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A151">
         <v>23</v>
       </c>
@@ -5836,7 +5846,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="152" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="152" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A152">
         <v>23</v>
       </c>
@@ -5871,7 +5881,7 @@
         <v>21253</v>
       </c>
     </row>
-    <row r="153" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="153" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A153">
         <v>23</v>
       </c>
@@ -5906,7 +5916,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="154" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="154" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A154">
         <v>23</v>
       </c>
@@ -5941,7 +5951,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="155" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="155" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A155">
         <v>23</v>
       </c>
@@ -5976,7 +5986,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="156" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="156" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A156">
         <v>23</v>
       </c>
@@ -6011,7 +6021,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="157" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="157" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A157">
         <v>23</v>
       </c>
@@ -6046,7 +6056,7 @@
         <v>21253</v>
       </c>
     </row>
-    <row r="158" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="158" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A158">
         <v>24</v>
       </c>
@@ -6081,7 +6091,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="159" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="159" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A159">
         <v>24</v>
       </c>
@@ -6116,7 +6126,7 @@
         <v>11786</v>
       </c>
     </row>
-    <row r="160" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="160" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A160">
         <v>24</v>
       </c>
@@ -6151,7 +6161,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="161" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="161" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A161">
         <v>24</v>
       </c>
@@ -6186,7 +6196,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="162" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="162" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A162">
         <v>24</v>
       </c>
@@ -6221,7 +6231,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="163" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="163" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A163">
         <v>24</v>
       </c>
@@ -6256,7 +6266,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="164" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="164" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A164">
         <v>24</v>
       </c>
@@ -6289,6 +6299,496 @@
       </c>
       <c r="K164" s="1">
         <v>11786</v>
+      </c>
+    </row>
+    <row r="165" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A165">
+        <v>25</v>
+      </c>
+      <c r="B165" t="s">
+        <v>11</v>
+      </c>
+      <c r="C165">
+        <v>5</v>
+      </c>
+      <c r="D165">
+        <v>20</v>
+      </c>
+      <c r="E165">
+        <v>0</v>
+      </c>
+      <c r="F165">
+        <v>0</v>
+      </c>
+      <c r="G165">
+        <v>0</v>
+      </c>
+      <c r="H165" s="1">
+        <v>89814</v>
+      </c>
+      <c r="I165" t="s">
+        <v>12</v>
+      </c>
+      <c r="J165" t="s">
+        <v>13</v>
+      </c>
+      <c r="K165" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="166" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A166">
+        <v>25</v>
+      </c>
+      <c r="B166" t="s">
+        <v>14</v>
+      </c>
+      <c r="C166">
+        <v>4</v>
+      </c>
+      <c r="D166">
+        <v>12</v>
+      </c>
+      <c r="E166">
+        <v>4</v>
+      </c>
+      <c r="F166">
+        <v>0</v>
+      </c>
+      <c r="G166">
+        <v>0</v>
+      </c>
+      <c r="H166" s="1">
+        <v>59529</v>
+      </c>
+      <c r="I166" s="1">
+        <v>6550</v>
+      </c>
+      <c r="J166" s="1">
+        <v>1037</v>
+      </c>
+      <c r="K166" s="1">
+        <v>22385</v>
+      </c>
+    </row>
+    <row r="167" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A167">
+        <v>25</v>
+      </c>
+      <c r="B167" t="s">
+        <v>15</v>
+      </c>
+      <c r="C167">
+        <v>6</v>
+      </c>
+      <c r="D167">
+        <v>24</v>
+      </c>
+      <c r="E167">
+        <v>0</v>
+      </c>
+      <c r="F167">
+        <v>0</v>
+      </c>
+      <c r="G167">
+        <v>0</v>
+      </c>
+      <c r="H167" s="1">
+        <v>90014</v>
+      </c>
+      <c r="I167" t="s">
+        <v>12</v>
+      </c>
+      <c r="J167" t="s">
+        <v>13</v>
+      </c>
+      <c r="K167" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="168" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A168">
+        <v>25</v>
+      </c>
+      <c r="B168" t="s">
+        <v>16</v>
+      </c>
+      <c r="C168">
+        <v>6</v>
+      </c>
+      <c r="D168">
+        <v>24</v>
+      </c>
+      <c r="E168">
+        <v>0</v>
+      </c>
+      <c r="F168">
+        <v>0</v>
+      </c>
+      <c r="G168">
+        <v>0</v>
+      </c>
+      <c r="H168" s="1">
+        <v>78675</v>
+      </c>
+      <c r="I168" t="s">
+        <v>12</v>
+      </c>
+      <c r="J168" t="s">
+        <v>13</v>
+      </c>
+      <c r="K168" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="169" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A169">
+        <v>25</v>
+      </c>
+      <c r="B169" t="s">
+        <v>17</v>
+      </c>
+      <c r="C169">
+        <v>6</v>
+      </c>
+      <c r="D169">
+        <v>24</v>
+      </c>
+      <c r="E169">
+        <v>0</v>
+      </c>
+      <c r="F169">
+        <v>0</v>
+      </c>
+      <c r="G169">
+        <v>0</v>
+      </c>
+      <c r="H169" s="1">
+        <v>89853</v>
+      </c>
+      <c r="I169" t="s">
+        <v>12</v>
+      </c>
+      <c r="J169" t="s">
+        <v>13</v>
+      </c>
+      <c r="K169" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="170" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A170">
+        <v>25</v>
+      </c>
+      <c r="B170" t="s">
+        <v>18</v>
+      </c>
+      <c r="C170">
+        <v>6</v>
+      </c>
+      <c r="D170">
+        <v>24</v>
+      </c>
+      <c r="E170">
+        <v>0</v>
+      </c>
+      <c r="F170">
+        <v>0</v>
+      </c>
+      <c r="G170">
+        <v>0</v>
+      </c>
+      <c r="H170" s="1">
+        <v>81796</v>
+      </c>
+      <c r="I170" t="s">
+        <v>12</v>
+      </c>
+      <c r="J170" t="s">
+        <v>13</v>
+      </c>
+      <c r="K170" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="171" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A171">
+        <v>25</v>
+      </c>
+      <c r="B171" t="s">
+        <v>19</v>
+      </c>
+      <c r="C171">
+        <v>33</v>
+      </c>
+      <c r="D171">
+        <v>128</v>
+      </c>
+      <c r="E171">
+        <v>4</v>
+      </c>
+      <c r="F171">
+        <v>0</v>
+      </c>
+      <c r="G171">
+        <v>0</v>
+      </c>
+      <c r="H171" s="1">
+        <v>489681</v>
+      </c>
+      <c r="I171" s="1">
+        <v>6550</v>
+      </c>
+      <c r="J171" s="1">
+        <v>1037</v>
+      </c>
+      <c r="K171" s="1">
+        <v>22385</v>
+      </c>
+    </row>
+    <row r="172" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A172">
+        <v>26</v>
+      </c>
+      <c r="B172" t="s">
+        <v>11</v>
+      </c>
+      <c r="C172">
+        <v>5</v>
+      </c>
+      <c r="D172">
+        <v>20</v>
+      </c>
+      <c r="E172">
+        <v>0</v>
+      </c>
+      <c r="F172">
+        <v>0</v>
+      </c>
+      <c r="G172">
+        <v>0</v>
+      </c>
+      <c r="H172" s="1">
+        <v>81287</v>
+      </c>
+      <c r="I172" t="s">
+        <v>12</v>
+      </c>
+      <c r="J172" t="s">
+        <v>13</v>
+      </c>
+      <c r="K172" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="173" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A173">
+        <v>26</v>
+      </c>
+      <c r="B173" t="s">
+        <v>14</v>
+      </c>
+      <c r="C173">
+        <v>6</v>
+      </c>
+      <c r="D173">
+        <v>24</v>
+      </c>
+      <c r="E173">
+        <v>0</v>
+      </c>
+      <c r="F173">
+        <v>0</v>
+      </c>
+      <c r="G173">
+        <v>0</v>
+      </c>
+      <c r="H173" s="1">
+        <v>93832</v>
+      </c>
+      <c r="I173" t="s">
+        <v>12</v>
+      </c>
+      <c r="J173" t="s">
+        <v>13</v>
+      </c>
+      <c r="K173" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="174" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A174">
+        <v>26</v>
+      </c>
+      <c r="B174" t="s">
+        <v>15</v>
+      </c>
+      <c r="C174">
+        <v>6</v>
+      </c>
+      <c r="D174">
+        <v>24</v>
+      </c>
+      <c r="E174">
+        <v>0</v>
+      </c>
+      <c r="F174">
+        <v>0</v>
+      </c>
+      <c r="G174">
+        <v>0</v>
+      </c>
+      <c r="H174" s="1">
+        <v>86343</v>
+      </c>
+      <c r="I174" t="s">
+        <v>12</v>
+      </c>
+      <c r="J174" t="s">
+        <v>13</v>
+      </c>
+      <c r="K174" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="175" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A175">
+        <v>26</v>
+      </c>
+      <c r="B175" t="s">
+        <v>16</v>
+      </c>
+      <c r="C175">
+        <v>6</v>
+      </c>
+      <c r="D175">
+        <v>24</v>
+      </c>
+      <c r="E175">
+        <v>0</v>
+      </c>
+      <c r="F175">
+        <v>0</v>
+      </c>
+      <c r="G175">
+        <v>0</v>
+      </c>
+      <c r="H175" s="1">
+        <v>79748</v>
+      </c>
+      <c r="I175" t="s">
+        <v>12</v>
+      </c>
+      <c r="J175" t="s">
+        <v>13</v>
+      </c>
+      <c r="K175" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="176" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A176">
+        <v>26</v>
+      </c>
+      <c r="B176" t="s">
+        <v>17</v>
+      </c>
+      <c r="C176">
+        <v>6</v>
+      </c>
+      <c r="D176">
+        <v>24</v>
+      </c>
+      <c r="E176">
+        <v>0</v>
+      </c>
+      <c r="F176">
+        <v>0</v>
+      </c>
+      <c r="G176">
+        <v>0</v>
+      </c>
+      <c r="H176" s="1">
+        <v>83488</v>
+      </c>
+      <c r="I176" t="s">
+        <v>12</v>
+      </c>
+      <c r="J176" t="s">
+        <v>13</v>
+      </c>
+      <c r="K176" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="177" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A177">
+        <v>26</v>
+      </c>
+      <c r="B177" t="s">
+        <v>18</v>
+      </c>
+      <c r="C177">
+        <v>6</v>
+      </c>
+      <c r="D177">
+        <v>24</v>
+      </c>
+      <c r="E177">
+        <v>0</v>
+      </c>
+      <c r="F177">
+        <v>0</v>
+      </c>
+      <c r="G177">
+        <v>0</v>
+      </c>
+      <c r="H177" s="1">
+        <v>81827</v>
+      </c>
+      <c r="I177" t="s">
+        <v>12</v>
+      </c>
+      <c r="J177" t="s">
+        <v>13</v>
+      </c>
+      <c r="K177" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="178" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A178">
+        <v>26</v>
+      </c>
+      <c r="B178" t="s">
+        <v>19</v>
+      </c>
+      <c r="C178">
+        <v>35</v>
+      </c>
+      <c r="D178">
+        <v>140</v>
+      </c>
+      <c r="E178">
+        <v>0</v>
+      </c>
+      <c r="F178">
+        <v>0</v>
+      </c>
+      <c r="G178">
+        <v>0</v>
+      </c>
+      <c r="H178" s="1">
+        <v>506525</v>
+      </c>
+      <c r="I178" t="s">
+        <v>12</v>
+      </c>
+      <c r="J178" t="s">
+        <v>13</v>
+      </c>
+      <c r="K178" t="s">
+        <v>13</v>
       </c>
     </row>
   </sheetData>
@@ -6299,14 +6799,14 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DC5A6928-3806-4082-94AB-A52936AB7317}">
-  <dimension ref="A1:B25"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:B27"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="27.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="5.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="27.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -6314,7 +6814,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>1</v>
       </c>
@@ -6322,7 +6822,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>2</v>
       </c>
@@ -6330,7 +6830,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>3</v>
       </c>
@@ -6338,7 +6838,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>4</v>
       </c>
@@ -6346,7 +6846,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>5</v>
       </c>
@@ -6354,7 +6854,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>6</v>
       </c>
@@ -6362,7 +6862,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>7</v>
       </c>
@@ -6370,7 +6870,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>8</v>
       </c>
@@ -6378,7 +6878,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>9</v>
       </c>
@@ -6386,7 +6886,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>10</v>
       </c>
@@ -6394,7 +6894,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A12">
         <v>11</v>
       </c>
@@ -6402,7 +6902,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>12</v>
       </c>
@@ -6410,7 +6910,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A14">
         <v>13</v>
       </c>
@@ -6418,7 +6918,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A15">
         <v>14</v>
       </c>
@@ -6426,7 +6926,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A16">
         <v>15</v>
       </c>
@@ -6434,7 +6934,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A17">
         <v>16</v>
       </c>
@@ -6442,7 +6942,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A18">
         <v>17</v>
       </c>
@@ -6450,7 +6950,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A19">
         <v>18</v>
       </c>
@@ -6458,7 +6958,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A20">
         <v>19</v>
       </c>
@@ -6466,7 +6966,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A21">
         <v>20</v>
       </c>
@@ -6474,7 +6974,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A22">
         <v>21</v>
       </c>
@@ -6482,7 +6982,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A23">
         <v>22</v>
       </c>
@@ -6490,7 +6990,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A24">
         <v>23</v>
       </c>
@@ -6498,12 +6998,28 @@
         <v>43</v>
       </c>
     </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A25">
         <v>24</v>
       </c>
       <c r="B25" t="s">
         <v>44</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A26">
+        <v>25</v>
+      </c>
+      <c r="B26" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A27">
+        <v>26</v>
+      </c>
+      <c r="B27" t="s">
+        <v>46</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Updated data files as of 12/15/25
</commit_message>
<xml_diff>
--- a/data_raw/smelt/abundance_estimates.xlsx
+++ b/data_raw/smelt/abundance_estimates.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://doimspp-my.sharepoint.com/personal/geasterbrook_usbr_gov/Documents/My Projects/SMT/Assessment/samt_smt_assessments-main/samt_smt_assessments-main/data_raw/smelt/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://doimspp-my.sharepoint.com/personal/lmccormick_usbr_gov/Documents/Documents/Research/R/samt_smt_assessments/data_raw/smelt/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="57" documentId="8_{BF3B047A-36C0-4AD4-A0BA-7FD3D60567F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C5C37F8A-FBC3-4F0E-B638-1EE44A59CD0A}"/>
+  <xr:revisionPtr revIDLastSave="63" documentId="8_{BF3B047A-36C0-4AD4-A0BA-7FD3D60567F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0680A420-3847-4C6C-8136-85EB3CC4707E}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{03E7A685-4EE0-4A4E-B4B4-B1F660F8462C}"/>
+    <workbookView xWindow="11508" yWindow="-14616" windowWidth="24972" windowHeight="13260" xr2:uid="{03E7A685-4EE0-4A4E-B4B4-B1F660F8462C}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="24">
   <si>
     <t>Week</t>
   </si>
@@ -106,13 +106,16 @@
   </si>
   <si>
     <t>Southern Delta</t>
+  </si>
+  <si>
+    <t>December 8–12, 2025</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -120,25 +123,13 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF000000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFFF"/>
-        <bgColor indexed="64"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -153,21 +144,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="3" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -506,14 +485,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{91E6CDBE-81F8-437E-8236-059C4BBF9395}">
-  <dimension ref="A1:K9"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:K17"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="19.90625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="16.36328125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="19.88671875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="16.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -548,284 +527,564 @@
         <v>10</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A2" s="4">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A2">
         <v>1</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B2" t="s">
         <v>11</v>
       </c>
-      <c r="C2" s="4">
+      <c r="C2">
         <v>6</v>
       </c>
-      <c r="D2" s="4">
+      <c r="D2">
         <v>24</v>
       </c>
-      <c r="E2" s="4">
-        <v>0</v>
-      </c>
-      <c r="F2" s="4">
-        <v>0</v>
-      </c>
-      <c r="G2" s="4">
-        <v>0</v>
-      </c>
-      <c r="H2" s="5">
+      <c r="E2">
+        <v>0</v>
+      </c>
+      <c r="F2">
+        <v>0</v>
+      </c>
+      <c r="G2">
+        <v>0</v>
+      </c>
+      <c r="H2">
         <v>105423</v>
       </c>
-      <c r="I2" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="J2" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="K2" s="4" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A3" s="4">
+      <c r="I2" t="s">
+        <v>12</v>
+      </c>
+      <c r="J2" t="s">
+        <v>13</v>
+      </c>
+      <c r="K2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A3">
         <v>1</v>
       </c>
-      <c r="B3" s="1" t="s">
+      <c r="B3" t="s">
         <v>14</v>
       </c>
-      <c r="C3" s="4">
+      <c r="C3">
         <v>3</v>
       </c>
-      <c r="D3" s="4">
+      <c r="D3">
         <v>10</v>
       </c>
-      <c r="E3" s="4">
+      <c r="E3">
         <v>1</v>
       </c>
-      <c r="F3" s="4">
-        <v>0</v>
-      </c>
-      <c r="G3" s="4">
-        <v>0</v>
-      </c>
-      <c r="H3" s="5">
+      <c r="F3">
+        <v>0</v>
+      </c>
+      <c r="G3">
+        <v>0</v>
+      </c>
+      <c r="H3">
         <v>36433</v>
       </c>
-      <c r="I3" s="5">
+      <c r="I3">
         <v>2413</v>
       </c>
-      <c r="J3" s="4">
+      <c r="J3">
         <v>186</v>
       </c>
-      <c r="K3" s="5">
+      <c r="K3">
         <v>10740</v>
       </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A4" s="4">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A4">
         <v>1</v>
       </c>
-      <c r="B4" s="1" t="s">
+      <c r="B4" t="s">
         <v>15</v>
       </c>
-      <c r="C4" s="4">
+      <c r="C4">
         <v>3</v>
       </c>
-      <c r="D4" s="4">
-        <v>12</v>
-      </c>
-      <c r="E4" s="4">
-        <v>0</v>
-      </c>
-      <c r="F4" s="4">
-        <v>0</v>
-      </c>
-      <c r="G4" s="4">
-        <v>0</v>
-      </c>
-      <c r="H4" s="5">
+      <c r="D4">
+        <v>12</v>
+      </c>
+      <c r="E4">
+        <v>0</v>
+      </c>
+      <c r="F4">
+        <v>0</v>
+      </c>
+      <c r="G4">
+        <v>0</v>
+      </c>
+      <c r="H4">
         <v>45635</v>
       </c>
-      <c r="I4" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="J4" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="K4" s="4" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A5" s="4">
+      <c r="I4" t="s">
+        <v>12</v>
+      </c>
+      <c r="J4" t="s">
+        <v>13</v>
+      </c>
+      <c r="K4" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A5">
         <v>1</v>
       </c>
-      <c r="B5" s="1" t="s">
+      <c r="B5" t="s">
         <v>16</v>
       </c>
-      <c r="C5" s="4">
+      <c r="C5">
         <v>3</v>
       </c>
-      <c r="D5" s="4">
+      <c r="D5">
         <v>10</v>
       </c>
-      <c r="E5" s="4">
-        <v>0</v>
-      </c>
-      <c r="F5" s="4">
-        <v>0</v>
-      </c>
-      <c r="G5" s="4">
-        <v>0</v>
-      </c>
-      <c r="H5" s="5">
+      <c r="E5">
+        <v>0</v>
+      </c>
+      <c r="F5">
+        <v>0</v>
+      </c>
+      <c r="G5">
+        <v>0</v>
+      </c>
+      <c r="H5">
         <v>34251</v>
       </c>
-      <c r="I5" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="J5" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="K5" s="4" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A6" s="4">
+      <c r="I5" t="s">
+        <v>12</v>
+      </c>
+      <c r="J5" t="s">
+        <v>13</v>
+      </c>
+      <c r="K5" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A6">
         <v>1</v>
       </c>
-      <c r="B6" s="1" t="s">
+      <c r="B6" t="s">
         <v>17</v>
       </c>
-      <c r="C6" s="4">
+      <c r="C6">
         <v>3</v>
       </c>
-      <c r="D6" s="4">
-        <v>12</v>
-      </c>
-      <c r="E6" s="4">
+      <c r="D6">
+        <v>12</v>
+      </c>
+      <c r="E6">
         <v>1</v>
       </c>
-      <c r="F6" s="4">
-        <v>0</v>
-      </c>
-      <c r="G6" s="4">
-        <v>0</v>
-      </c>
-      <c r="H6" s="5">
+      <c r="F6">
+        <v>0</v>
+      </c>
+      <c r="G6">
+        <v>0</v>
+      </c>
+      <c r="H6">
         <v>47846</v>
       </c>
-      <c r="I6" s="4">
+      <c r="I6">
         <v>693</v>
       </c>
-      <c r="J6" s="4">
+      <c r="J6">
         <v>54</v>
       </c>
-      <c r="K6" s="5">
+      <c r="K6">
         <v>3065</v>
       </c>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A7" s="4">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A7">
         <v>1</v>
       </c>
-      <c r="B7" s="1" t="s">
+      <c r="B7" t="s">
         <v>18</v>
       </c>
-      <c r="C7" s="4">
+      <c r="C7">
         <v>6</v>
       </c>
-      <c r="D7" s="4">
+      <c r="D7">
         <v>24</v>
       </c>
-      <c r="E7" s="4">
-        <v>0</v>
-      </c>
-      <c r="F7" s="4">
-        <v>0</v>
-      </c>
-      <c r="G7" s="4">
-        <v>0</v>
-      </c>
-      <c r="H7" s="5">
+      <c r="E7">
+        <v>0</v>
+      </c>
+      <c r="F7">
+        <v>0</v>
+      </c>
+      <c r="G7">
+        <v>0</v>
+      </c>
+      <c r="H7">
         <v>96303</v>
       </c>
-      <c r="I7" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="J7" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="K7" s="4" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A8" s="4">
+      <c r="I7" t="s">
+        <v>12</v>
+      </c>
+      <c r="J7" t="s">
+        <v>13</v>
+      </c>
+      <c r="K7" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A8">
         <v>1</v>
       </c>
-      <c r="B8" s="1" t="s">
+      <c r="B8" t="s">
         <v>22</v>
       </c>
-      <c r="C8" s="4">
+      <c r="C8">
         <v>3</v>
       </c>
-      <c r="D8" s="4">
-        <v>12</v>
-      </c>
-      <c r="E8" s="4">
-        <v>0</v>
-      </c>
-      <c r="F8" s="4">
-        <v>0</v>
-      </c>
-      <c r="G8" s="4">
-        <v>0</v>
-      </c>
-      <c r="H8" s="5">
+      <c r="D8">
+        <v>12</v>
+      </c>
+      <c r="E8">
+        <v>0</v>
+      </c>
+      <c r="F8">
+        <v>0</v>
+      </c>
+      <c r="G8">
+        <v>0</v>
+      </c>
+      <c r="H8">
         <v>39136</v>
       </c>
-      <c r="I8" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="J8" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="K8" s="4" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A9" s="4">
+      <c r="I8" t="s">
+        <v>12</v>
+      </c>
+      <c r="J8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K8" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A9">
         <v>1</v>
       </c>
-      <c r="B9" s="1" t="s">
+      <c r="B9" t="s">
         <v>19</v>
       </c>
-      <c r="C9" s="4">
+      <c r="C9">
         <v>27</v>
       </c>
-      <c r="D9" s="4">
+      <c r="D9">
         <v>104</v>
       </c>
-      <c r="E9" s="4">
+      <c r="E9">
         <v>2</v>
       </c>
-      <c r="F9" s="4">
-        <v>0</v>
-      </c>
-      <c r="G9" s="4">
-        <v>0</v>
-      </c>
-      <c r="H9" s="5">
+      <c r="F9">
+        <v>0</v>
+      </c>
+      <c r="G9">
+        <v>0</v>
+      </c>
+      <c r="H9">
         <v>405027</v>
       </c>
-      <c r="I9" s="5">
+      <c r="I9">
         <v>3106</v>
       </c>
-      <c r="J9" s="4">
+      <c r="J9">
         <v>354</v>
       </c>
-      <c r="K9" s="5">
+      <c r="K9">
         <v>12103</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A10">
+        <v>2</v>
+      </c>
+      <c r="B10" t="s">
+        <v>11</v>
+      </c>
+      <c r="C10">
+        <v>6</v>
+      </c>
+      <c r="D10">
+        <v>24</v>
+      </c>
+      <c r="E10">
+        <v>0</v>
+      </c>
+      <c r="F10">
+        <v>0</v>
+      </c>
+      <c r="G10">
+        <v>0</v>
+      </c>
+      <c r="H10" s="1">
+        <v>95805</v>
+      </c>
+      <c r="I10" t="s">
+        <v>12</v>
+      </c>
+      <c r="J10" t="s">
+        <v>13</v>
+      </c>
+      <c r="K10" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A11">
+        <v>2</v>
+      </c>
+      <c r="B11" t="s">
+        <v>14</v>
+      </c>
+      <c r="C11">
+        <v>6</v>
+      </c>
+      <c r="D11">
+        <v>18</v>
+      </c>
+      <c r="E11">
+        <v>8</v>
+      </c>
+      <c r="F11">
+        <v>0</v>
+      </c>
+      <c r="G11">
+        <v>0</v>
+      </c>
+      <c r="H11" s="1">
+        <v>71780</v>
+      </c>
+      <c r="I11" s="1">
+        <v>10092</v>
+      </c>
+      <c r="J11" s="1">
+        <v>2302</v>
+      </c>
+      <c r="K11" s="1">
+        <v>29101</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A12">
+        <v>2</v>
+      </c>
+      <c r="B12" t="s">
+        <v>15</v>
+      </c>
+      <c r="C12">
+        <v>6</v>
+      </c>
+      <c r="D12">
+        <v>24</v>
+      </c>
+      <c r="E12">
+        <v>0</v>
+      </c>
+      <c r="F12">
+        <v>0</v>
+      </c>
+      <c r="G12">
+        <v>0</v>
+      </c>
+      <c r="H12" s="1">
+        <v>90024</v>
+      </c>
+      <c r="I12" t="s">
+        <v>12</v>
+      </c>
+      <c r="J12" t="s">
+        <v>13</v>
+      </c>
+      <c r="K12" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A13">
+        <v>2</v>
+      </c>
+      <c r="B13" t="s">
+        <v>16</v>
+      </c>
+      <c r="C13">
+        <v>3</v>
+      </c>
+      <c r="D13">
+        <v>12</v>
+      </c>
+      <c r="E13">
+        <v>0</v>
+      </c>
+      <c r="F13">
+        <v>0</v>
+      </c>
+      <c r="G13">
+        <v>0</v>
+      </c>
+      <c r="H13" s="1">
+        <v>40984</v>
+      </c>
+      <c r="I13" t="s">
+        <v>12</v>
+      </c>
+      <c r="J13" t="s">
+        <v>13</v>
+      </c>
+      <c r="K13" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A14">
+        <v>2</v>
+      </c>
+      <c r="B14" t="s">
+        <v>17</v>
+      </c>
+      <c r="C14">
+        <v>3</v>
+      </c>
+      <c r="D14">
+        <v>12</v>
+      </c>
+      <c r="E14">
+        <v>0</v>
+      </c>
+      <c r="F14">
+        <v>0</v>
+      </c>
+      <c r="G14">
+        <v>0</v>
+      </c>
+      <c r="H14" s="1">
+        <v>41168</v>
+      </c>
+      <c r="I14" t="s">
+        <v>12</v>
+      </c>
+      <c r="J14" t="s">
+        <v>13</v>
+      </c>
+      <c r="K14" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A15">
+        <v>2</v>
+      </c>
+      <c r="B15" t="s">
+        <v>18</v>
+      </c>
+      <c r="C15">
+        <v>6</v>
+      </c>
+      <c r="D15">
+        <v>24</v>
+      </c>
+      <c r="E15">
+        <v>0</v>
+      </c>
+      <c r="F15">
+        <v>0</v>
+      </c>
+      <c r="G15">
+        <v>0</v>
+      </c>
+      <c r="H15" s="1">
+        <v>89940</v>
+      </c>
+      <c r="I15" t="s">
+        <v>12</v>
+      </c>
+      <c r="J15" t="s">
+        <v>13</v>
+      </c>
+      <c r="K15" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A16">
+        <v>2</v>
+      </c>
+      <c r="B16" t="s">
+        <v>22</v>
+      </c>
+      <c r="C16">
+        <v>5</v>
+      </c>
+      <c r="D16">
+        <v>20</v>
+      </c>
+      <c r="E16">
+        <v>0</v>
+      </c>
+      <c r="F16">
+        <v>0</v>
+      </c>
+      <c r="G16">
+        <v>0</v>
+      </c>
+      <c r="H16" s="1">
+        <v>73402</v>
+      </c>
+      <c r="I16" t="s">
+        <v>12</v>
+      </c>
+      <c r="J16" t="s">
+        <v>13</v>
+      </c>
+      <c r="K16" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A17">
+        <v>2</v>
+      </c>
+      <c r="B17" t="s">
+        <v>19</v>
+      </c>
+      <c r="C17">
+        <v>35</v>
+      </c>
+      <c r="D17">
+        <v>134</v>
+      </c>
+      <c r="E17">
+        <v>8</v>
+      </c>
+      <c r="F17">
+        <v>0</v>
+      </c>
+      <c r="G17">
+        <v>0</v>
+      </c>
+      <c r="H17" s="1">
+        <v>503104</v>
+      </c>
+      <c r="I17" s="1">
+        <v>10092</v>
+      </c>
+      <c r="J17" s="1">
+        <v>2302</v>
+      </c>
+      <c r="K17" s="1">
+        <v>29101</v>
       </c>
     </row>
   </sheetData>
@@ -836,52 +1095,36 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DC5A6928-3806-4082-94AB-A52936AB7317}">
-  <dimension ref="A1:B8"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:B3"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="5.6328125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="27.54296875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="5.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="27.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A1" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="2" t="s">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A2" s="2">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A2">
         <v>1</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="B2" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A3" s="2"/>
-      <c r="B3" s="2"/>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A4" s="2"/>
-      <c r="B4" s="2"/>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A5" s="2"/>
-      <c r="B5" s="2"/>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A6" s="2"/>
-      <c r="B6" s="2"/>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A7" s="2"/>
-      <c r="B7" s="2"/>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A8" s="2"/>
-      <c r="B8" s="2"/>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3" t="s">
+        <v>23</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Edits for 12/30 smelt assessment. Updated catch code, added beach seine, added bay study
</commit_message>
<xml_diff>
--- a/data_raw/smelt/abundance_estimates.xlsx
+++ b/data_raw/smelt/abundance_estimates.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://doimspp-my.sharepoint.com/personal/lmccormick_usbr_gov/Documents/Documents/Research/R/samt_smt_assessments/data_raw/smelt/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="63" documentId="8_{BF3B047A-36C0-4AD4-A0BA-7FD3D60567F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0680A420-3847-4C6C-8136-85EB3CC4707E}"/>
+  <xr:revisionPtr revIDLastSave="71" documentId="8_{BF3B047A-36C0-4AD4-A0BA-7FD3D60567F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E892E23A-7D82-4D8D-8278-5646134FE0BD}"/>
   <bookViews>
-    <workbookView xWindow="11508" yWindow="-14616" windowWidth="24972" windowHeight="13260" xr2:uid="{03E7A685-4EE0-4A4E-B4B4-B1F660F8462C}"/>
+    <workbookView xWindow="15828" yWindow="-15300" windowWidth="23040" windowHeight="12120" xr2:uid="{03E7A685-4EE0-4A4E-B4B4-B1F660F8462C}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="118" uniqueCount="26">
   <si>
     <t>Week</t>
   </si>
@@ -109,6 +109,12 @@
   </si>
   <si>
     <t>December 8–12, 2025</t>
+  </si>
+  <si>
+    <t>December 15–19, 2025</t>
+  </si>
+  <si>
+    <t>December 21–26, 2025</t>
   </si>
 </sst>
 </file>
@@ -485,7 +491,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{91E6CDBE-81F8-437E-8236-059C4BBF9395}">
-  <dimension ref="A1:K17"/>
+  <dimension ref="A1:K33"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="19.88671875" bestFit="1" customWidth="1"/>
@@ -1087,6 +1093,566 @@
         <v>29101</v>
       </c>
     </row>
+    <row r="18" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A18">
+        <v>3</v>
+      </c>
+      <c r="B18" t="s">
+        <v>11</v>
+      </c>
+      <c r="C18">
+        <v>6</v>
+      </c>
+      <c r="D18">
+        <v>24</v>
+      </c>
+      <c r="E18">
+        <v>0</v>
+      </c>
+      <c r="F18">
+        <v>0</v>
+      </c>
+      <c r="G18">
+        <v>0</v>
+      </c>
+      <c r="H18" s="1">
+        <v>92752</v>
+      </c>
+      <c r="I18" t="s">
+        <v>12</v>
+      </c>
+      <c r="J18" t="s">
+        <v>13</v>
+      </c>
+      <c r="K18" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="19" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A19">
+        <v>3</v>
+      </c>
+      <c r="B19" t="s">
+        <v>14</v>
+      </c>
+      <c r="C19">
+        <v>6</v>
+      </c>
+      <c r="D19">
+        <v>20</v>
+      </c>
+      <c r="E19">
+        <v>2</v>
+      </c>
+      <c r="F19">
+        <v>0</v>
+      </c>
+      <c r="G19">
+        <v>0</v>
+      </c>
+      <c r="H19" s="1">
+        <v>77481</v>
+      </c>
+      <c r="I19" s="1">
+        <v>2515</v>
+      </c>
+      <c r="J19">
+        <v>373</v>
+      </c>
+      <c r="K19" s="1">
+        <v>8836</v>
+      </c>
+    </row>
+    <row r="20" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A20">
+        <v>3</v>
+      </c>
+      <c r="B20" t="s">
+        <v>15</v>
+      </c>
+      <c r="C20">
+        <v>6</v>
+      </c>
+      <c r="D20">
+        <v>24</v>
+      </c>
+      <c r="E20">
+        <v>0</v>
+      </c>
+      <c r="F20">
+        <v>0</v>
+      </c>
+      <c r="G20">
+        <v>0</v>
+      </c>
+      <c r="H20" s="1">
+        <v>84555</v>
+      </c>
+      <c r="I20" t="s">
+        <v>12</v>
+      </c>
+      <c r="J20" t="s">
+        <v>13</v>
+      </c>
+      <c r="K20" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="21" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A21">
+        <v>3</v>
+      </c>
+      <c r="B21" t="s">
+        <v>16</v>
+      </c>
+      <c r="C21">
+        <v>3</v>
+      </c>
+      <c r="D21">
+        <v>12</v>
+      </c>
+      <c r="E21">
+        <v>0</v>
+      </c>
+      <c r="F21">
+        <v>0</v>
+      </c>
+      <c r="G21">
+        <v>0</v>
+      </c>
+      <c r="H21" s="1">
+        <v>38298</v>
+      </c>
+      <c r="I21" t="s">
+        <v>12</v>
+      </c>
+      <c r="J21" t="s">
+        <v>13</v>
+      </c>
+      <c r="K21" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="22" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A22">
+        <v>3</v>
+      </c>
+      <c r="B22" t="s">
+        <v>17</v>
+      </c>
+      <c r="C22">
+        <v>3</v>
+      </c>
+      <c r="D22">
+        <v>12</v>
+      </c>
+      <c r="E22">
+        <v>0</v>
+      </c>
+      <c r="F22">
+        <v>0</v>
+      </c>
+      <c r="G22">
+        <v>0</v>
+      </c>
+      <c r="H22" s="1">
+        <v>42242</v>
+      </c>
+      <c r="I22" t="s">
+        <v>12</v>
+      </c>
+      <c r="J22" t="s">
+        <v>13</v>
+      </c>
+      <c r="K22" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="23" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A23">
+        <v>3</v>
+      </c>
+      <c r="B23" t="s">
+        <v>18</v>
+      </c>
+      <c r="C23">
+        <v>6</v>
+      </c>
+      <c r="D23">
+        <v>24</v>
+      </c>
+      <c r="E23">
+        <v>0</v>
+      </c>
+      <c r="F23">
+        <v>0</v>
+      </c>
+      <c r="G23">
+        <v>0</v>
+      </c>
+      <c r="H23" s="1">
+        <v>88641</v>
+      </c>
+      <c r="I23" t="s">
+        <v>12</v>
+      </c>
+      <c r="J23" t="s">
+        <v>13</v>
+      </c>
+      <c r="K23" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="24" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A24">
+        <v>3</v>
+      </c>
+      <c r="B24" t="s">
+        <v>22</v>
+      </c>
+      <c r="C24">
+        <v>5</v>
+      </c>
+      <c r="D24">
+        <v>20</v>
+      </c>
+      <c r="E24">
+        <v>0</v>
+      </c>
+      <c r="F24">
+        <v>0</v>
+      </c>
+      <c r="G24">
+        <v>0</v>
+      </c>
+      <c r="H24" s="1">
+        <v>76676</v>
+      </c>
+      <c r="I24" t="s">
+        <v>12</v>
+      </c>
+      <c r="J24" t="s">
+        <v>13</v>
+      </c>
+      <c r="K24" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="25" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A25">
+        <v>3</v>
+      </c>
+      <c r="B25" t="s">
+        <v>19</v>
+      </c>
+      <c r="C25">
+        <v>35</v>
+      </c>
+      <c r="D25">
+        <v>136</v>
+      </c>
+      <c r="E25">
+        <v>2</v>
+      </c>
+      <c r="F25">
+        <v>0</v>
+      </c>
+      <c r="G25">
+        <v>0</v>
+      </c>
+      <c r="H25" s="1">
+        <v>500645</v>
+      </c>
+      <c r="I25" s="1">
+        <v>2515</v>
+      </c>
+      <c r="J25">
+        <v>373</v>
+      </c>
+      <c r="K25" s="1">
+        <v>8836</v>
+      </c>
+    </row>
+    <row r="26" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A26">
+        <v>4</v>
+      </c>
+      <c r="B26" t="s">
+        <v>11</v>
+      </c>
+      <c r="C26">
+        <v>5</v>
+      </c>
+      <c r="D26">
+        <v>20</v>
+      </c>
+      <c r="E26">
+        <v>0</v>
+      </c>
+      <c r="F26">
+        <v>0</v>
+      </c>
+      <c r="G26">
+        <v>0</v>
+      </c>
+      <c r="H26" s="1">
+        <v>86146</v>
+      </c>
+      <c r="I26" t="s">
+        <v>12</v>
+      </c>
+      <c r="J26" t="s">
+        <v>13</v>
+      </c>
+      <c r="K26" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="27" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A27">
+        <v>4</v>
+      </c>
+      <c r="B27" t="s">
+        <v>14</v>
+      </c>
+      <c r="C27">
+        <v>4</v>
+      </c>
+      <c r="D27">
+        <v>13</v>
+      </c>
+      <c r="E27">
+        <v>2</v>
+      </c>
+      <c r="F27">
+        <v>0</v>
+      </c>
+      <c r="G27">
+        <v>0</v>
+      </c>
+      <c r="H27" s="1">
+        <v>54867</v>
+      </c>
+      <c r="I27" s="1">
+        <v>3081</v>
+      </c>
+      <c r="J27">
+        <v>359</v>
+      </c>
+      <c r="K27" s="1">
+        <v>11902</v>
+      </c>
+    </row>
+    <row r="28" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A28">
+        <v>4</v>
+      </c>
+      <c r="B28" t="s">
+        <v>15</v>
+      </c>
+      <c r="C28">
+        <v>3</v>
+      </c>
+      <c r="D28">
+        <v>12</v>
+      </c>
+      <c r="E28">
+        <v>0</v>
+      </c>
+      <c r="F28">
+        <v>0</v>
+      </c>
+      <c r="G28">
+        <v>0</v>
+      </c>
+      <c r="H28" s="1">
+        <v>40797</v>
+      </c>
+      <c r="I28" t="s">
+        <v>12</v>
+      </c>
+      <c r="J28" t="s">
+        <v>13</v>
+      </c>
+      <c r="K28" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="29" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A29">
+        <v>4</v>
+      </c>
+      <c r="B29" t="s">
+        <v>16</v>
+      </c>
+      <c r="C29">
+        <v>0</v>
+      </c>
+      <c r="D29">
+        <v>0</v>
+      </c>
+      <c r="E29">
+        <v>0</v>
+      </c>
+      <c r="F29">
+        <v>0</v>
+      </c>
+      <c r="G29">
+        <v>0</v>
+      </c>
+      <c r="H29">
+        <v>0</v>
+      </c>
+      <c r="I29" t="s">
+        <v>13</v>
+      </c>
+      <c r="J29" t="s">
+        <v>13</v>
+      </c>
+      <c r="K29" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="30" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A30">
+        <v>4</v>
+      </c>
+      <c r="B30" t="s">
+        <v>17</v>
+      </c>
+      <c r="C30">
+        <v>3</v>
+      </c>
+      <c r="D30">
+        <v>12</v>
+      </c>
+      <c r="E30">
+        <v>0</v>
+      </c>
+      <c r="F30">
+        <v>0</v>
+      </c>
+      <c r="G30">
+        <v>0</v>
+      </c>
+      <c r="H30" s="1">
+        <v>43917</v>
+      </c>
+      <c r="I30" t="s">
+        <v>12</v>
+      </c>
+      <c r="J30" t="s">
+        <v>13</v>
+      </c>
+      <c r="K30" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="31" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A31">
+        <v>4</v>
+      </c>
+      <c r="B31" t="s">
+        <v>18</v>
+      </c>
+      <c r="C31">
+        <v>3</v>
+      </c>
+      <c r="D31">
+        <v>10</v>
+      </c>
+      <c r="E31">
+        <v>0</v>
+      </c>
+      <c r="F31">
+        <v>0</v>
+      </c>
+      <c r="G31">
+        <v>0</v>
+      </c>
+      <c r="H31" s="1">
+        <v>40426</v>
+      </c>
+      <c r="I31" t="s">
+        <v>12</v>
+      </c>
+      <c r="J31" t="s">
+        <v>13</v>
+      </c>
+      <c r="K31" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="32" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A32">
+        <v>4</v>
+      </c>
+      <c r="B32" t="s">
+        <v>22</v>
+      </c>
+      <c r="C32">
+        <v>3</v>
+      </c>
+      <c r="D32">
+        <v>12</v>
+      </c>
+      <c r="E32">
+        <v>0</v>
+      </c>
+      <c r="F32">
+        <v>0</v>
+      </c>
+      <c r="G32">
+        <v>0</v>
+      </c>
+      <c r="H32" s="1">
+        <v>44275</v>
+      </c>
+      <c r="I32" t="s">
+        <v>12</v>
+      </c>
+      <c r="J32" t="s">
+        <v>13</v>
+      </c>
+      <c r="K32" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="33" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A33">
+        <v>4</v>
+      </c>
+      <c r="B33" t="s">
+        <v>19</v>
+      </c>
+      <c r="C33">
+        <v>21</v>
+      </c>
+      <c r="D33">
+        <v>79</v>
+      </c>
+      <c r="E33">
+        <v>2</v>
+      </c>
+      <c r="F33">
+        <v>0</v>
+      </c>
+      <c r="G33">
+        <v>0</v>
+      </c>
+      <c r="H33" s="1">
+        <v>310429</v>
+      </c>
+      <c r="I33" s="1">
+        <v>3081</v>
+      </c>
+      <c r="J33">
+        <v>359</v>
+      </c>
+      <c r="K33" s="1">
+        <v>11902</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
@@ -1095,7 +1661,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DC5A6928-3806-4082-94AB-A52936AB7317}">
-  <dimension ref="A1:B3"/>
+  <dimension ref="A1:B5"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="5.6640625" bestFit="1" customWidth="1"/>
@@ -1126,6 +1692,22 @@
         <v>23</v>
       </c>
     </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5" t="s">
+        <v>25</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
Smelt assessment code updates and data for 1/5
</commit_message>
<xml_diff>
--- a/data_raw/smelt/abundance_estimates.xlsx
+++ b/data_raw/smelt/abundance_estimates.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://doimspp-my.sharepoint.com/personal/lmccormick_usbr_gov/Documents/Documents/Research/R/samt_smt_assessments/data_raw/smelt/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="71" documentId="8_{BF3B047A-36C0-4AD4-A0BA-7FD3D60567F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E892E23A-7D82-4D8D-8278-5646134FE0BD}"/>
+  <xr:revisionPtr revIDLastSave="75" documentId="8_{BF3B047A-36C0-4AD4-A0BA-7FD3D60567F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{38504F95-CD43-4714-B6BE-20E56365B0A1}"/>
   <bookViews>
-    <workbookView xWindow="15828" yWindow="-15300" windowWidth="23040" windowHeight="12120" xr2:uid="{03E7A685-4EE0-4A4E-B4B4-B1F660F8462C}"/>
+    <workbookView xWindow="-24225" yWindow="3390" windowWidth="21600" windowHeight="11235" xr2:uid="{03E7A685-4EE0-4A4E-B4B4-B1F660F8462C}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="118" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="145" uniqueCount="27">
   <si>
     <t>Week</t>
   </si>
@@ -115,6 +115,9 @@
   </si>
   <si>
     <t>December 21–26, 2025</t>
+  </si>
+  <si>
+    <t>December 29, 2025–January 2, 2026</t>
   </si>
 </sst>
 </file>
@@ -491,14 +494,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{91E6CDBE-81F8-437E-8236-059C4BBF9395}">
-  <dimension ref="A1:K33"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:K41"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="19.88671875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="16.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="19.85546875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="16.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -533,7 +536,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
@@ -568,7 +571,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>1</v>
       </c>
@@ -603,7 +606,7 @@
         <v>10740</v>
       </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>1</v>
       </c>
@@ -638,7 +641,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>1</v>
       </c>
@@ -673,7 +676,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>1</v>
       </c>
@@ -708,7 +711,7 @@
         <v>3065</v>
       </c>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>1</v>
       </c>
@@ -743,7 +746,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>1</v>
       </c>
@@ -778,7 +781,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>1</v>
       </c>
@@ -813,7 +816,7 @@
         <v>12103</v>
       </c>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>2</v>
       </c>
@@ -848,7 +851,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>2</v>
       </c>
@@ -883,7 +886,7 @@
         <v>29101</v>
       </c>
     </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>2</v>
       </c>
@@ -918,7 +921,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>2</v>
       </c>
@@ -953,7 +956,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>2</v>
       </c>
@@ -988,7 +991,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>2</v>
       </c>
@@ -1023,7 +1026,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>2</v>
       </c>
@@ -1058,7 +1061,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>2</v>
       </c>
@@ -1093,7 +1096,7 @@
         <v>29101</v>
       </c>
     </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>3</v>
       </c>
@@ -1128,7 +1131,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>3</v>
       </c>
@@ -1163,7 +1166,7 @@
         <v>8836</v>
       </c>
     </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>3</v>
       </c>
@@ -1198,7 +1201,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>3</v>
       </c>
@@ -1233,7 +1236,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>3</v>
       </c>
@@ -1268,7 +1271,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A23">
         <v>3</v>
       </c>
@@ -1303,7 +1306,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>3</v>
       </c>
@@ -1338,7 +1341,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A25">
         <v>3</v>
       </c>
@@ -1373,7 +1376,7 @@
         <v>8836</v>
       </c>
     </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A26">
         <v>4</v>
       </c>
@@ -1408,7 +1411,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A27">
         <v>4</v>
       </c>
@@ -1443,7 +1446,7 @@
         <v>11902</v>
       </c>
     </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A28">
         <v>4</v>
       </c>
@@ -1478,7 +1481,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="29" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A29">
         <v>4</v>
       </c>
@@ -1513,7 +1516,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="30" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A30">
         <v>4</v>
       </c>
@@ -1548,7 +1551,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="31" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A31">
         <v>4</v>
       </c>
@@ -1583,7 +1586,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="32" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A32">
         <v>4</v>
       </c>
@@ -1618,7 +1621,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="33" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A33">
         <v>4</v>
       </c>
@@ -1651,6 +1654,286 @@
       </c>
       <c r="K33" s="1">
         <v>11902</v>
+      </c>
+    </row>
+    <row r="34" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A34">
+        <v>5</v>
+      </c>
+      <c r="B34" t="s">
+        <v>11</v>
+      </c>
+      <c r="C34">
+        <v>4</v>
+      </c>
+      <c r="D34">
+        <v>14</v>
+      </c>
+      <c r="E34">
+        <v>0</v>
+      </c>
+      <c r="F34">
+        <v>0</v>
+      </c>
+      <c r="G34">
+        <v>0</v>
+      </c>
+      <c r="H34" s="1">
+        <v>61453</v>
+      </c>
+      <c r="I34" t="s">
+        <v>12</v>
+      </c>
+      <c r="J34" t="s">
+        <v>13</v>
+      </c>
+      <c r="K34" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="35" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A35">
+        <v>5</v>
+      </c>
+      <c r="B35" t="s">
+        <v>14</v>
+      </c>
+      <c r="C35">
+        <v>6</v>
+      </c>
+      <c r="D35">
+        <v>19</v>
+      </c>
+      <c r="E35">
+        <v>5</v>
+      </c>
+      <c r="F35">
+        <v>0</v>
+      </c>
+      <c r="G35">
+        <v>0</v>
+      </c>
+      <c r="H35" s="1">
+        <v>72458</v>
+      </c>
+      <c r="I35" s="1">
+        <v>6821</v>
+      </c>
+      <c r="J35" s="1">
+        <v>1477</v>
+      </c>
+      <c r="K35" s="1">
+        <v>20185</v>
+      </c>
+    </row>
+    <row r="36" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A36">
+        <v>5</v>
+      </c>
+      <c r="B36" t="s">
+        <v>15</v>
+      </c>
+      <c r="C36">
+        <v>3</v>
+      </c>
+      <c r="D36">
+        <v>12</v>
+      </c>
+      <c r="E36">
+        <v>0</v>
+      </c>
+      <c r="F36">
+        <v>0</v>
+      </c>
+      <c r="G36">
+        <v>0</v>
+      </c>
+      <c r="H36" s="1">
+        <v>41318</v>
+      </c>
+      <c r="I36" t="s">
+        <v>12</v>
+      </c>
+      <c r="J36" t="s">
+        <v>13</v>
+      </c>
+      <c r="K36" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="37" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A37">
+        <v>5</v>
+      </c>
+      <c r="B37" t="s">
+        <v>16</v>
+      </c>
+      <c r="C37">
+        <v>3</v>
+      </c>
+      <c r="D37">
+        <v>12</v>
+      </c>
+      <c r="E37">
+        <v>0</v>
+      </c>
+      <c r="F37">
+        <v>0</v>
+      </c>
+      <c r="G37">
+        <v>0</v>
+      </c>
+      <c r="H37" s="1">
+        <v>32641</v>
+      </c>
+      <c r="I37" t="s">
+        <v>12</v>
+      </c>
+      <c r="J37" t="s">
+        <v>13</v>
+      </c>
+      <c r="K37" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="38" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A38">
+        <v>5</v>
+      </c>
+      <c r="B38" t="s">
+        <v>17</v>
+      </c>
+      <c r="C38">
+        <v>3</v>
+      </c>
+      <c r="D38">
+        <v>12</v>
+      </c>
+      <c r="E38">
+        <v>0</v>
+      </c>
+      <c r="F38">
+        <v>0</v>
+      </c>
+      <c r="G38">
+        <v>0</v>
+      </c>
+      <c r="H38" s="1">
+        <v>47200</v>
+      </c>
+      <c r="I38" t="s">
+        <v>12</v>
+      </c>
+      <c r="J38" t="s">
+        <v>13</v>
+      </c>
+      <c r="K38" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="39" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A39">
+        <v>5</v>
+      </c>
+      <c r="B39" t="s">
+        <v>18</v>
+      </c>
+      <c r="C39">
+        <v>6</v>
+      </c>
+      <c r="D39">
+        <v>24</v>
+      </c>
+      <c r="E39">
+        <v>0</v>
+      </c>
+      <c r="F39">
+        <v>0</v>
+      </c>
+      <c r="G39">
+        <v>0</v>
+      </c>
+      <c r="H39" s="1">
+        <v>83450</v>
+      </c>
+      <c r="I39" t="s">
+        <v>12</v>
+      </c>
+      <c r="J39" t="s">
+        <v>13</v>
+      </c>
+      <c r="K39" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="40" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A40">
+        <v>5</v>
+      </c>
+      <c r="B40" t="s">
+        <v>22</v>
+      </c>
+      <c r="C40">
+        <v>3</v>
+      </c>
+      <c r="D40">
+        <v>12</v>
+      </c>
+      <c r="E40">
+        <v>0</v>
+      </c>
+      <c r="F40">
+        <v>0</v>
+      </c>
+      <c r="G40">
+        <v>0</v>
+      </c>
+      <c r="H40" s="1">
+        <v>43567</v>
+      </c>
+      <c r="I40" t="s">
+        <v>12</v>
+      </c>
+      <c r="J40" t="s">
+        <v>13</v>
+      </c>
+      <c r="K40" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="41" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A41">
+        <v>5</v>
+      </c>
+      <c r="B41" t="s">
+        <v>19</v>
+      </c>
+      <c r="C41">
+        <v>28</v>
+      </c>
+      <c r="D41">
+        <v>105</v>
+      </c>
+      <c r="E41">
+        <v>5</v>
+      </c>
+      <c r="F41">
+        <v>0</v>
+      </c>
+      <c r="G41">
+        <v>0</v>
+      </c>
+      <c r="H41" s="1">
+        <v>382087</v>
+      </c>
+      <c r="I41" s="1">
+        <v>6821</v>
+      </c>
+      <c r="J41" s="1">
+        <v>1477</v>
+      </c>
+      <c r="K41" s="1">
+        <v>20185</v>
       </c>
     </row>
   </sheetData>
@@ -1661,14 +1944,14 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DC5A6928-3806-4082-94AB-A52936AB7317}">
-  <dimension ref="A1:B5"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:B6"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="5.6640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="27.5546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="5.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="27.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1676,7 +1959,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
@@ -1684,7 +1967,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2</v>
       </c>
@@ -1692,7 +1975,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>3</v>
       </c>
@@ -1700,12 +1983,20 @@
         <v>24</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>4</v>
       </c>
       <c r="B5" t="s">
         <v>25</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6" t="s">
+        <v>26</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
updated edsm abundance estimates 1/26
</commit_message>
<xml_diff>
--- a/data_raw/smelt/abundance_estimates.xlsx
+++ b/data_raw/smelt/abundance_estimates.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://doimspp-my.sharepoint.com/personal/geasterbrook_usbr_gov/Documents/My Projects/SMT/Assessment/samt_smt_assessments/data_raw/smelt/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="79" documentId="8_{BF3B047A-36C0-4AD4-A0BA-7FD3D60567F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{97FD1B19-9E17-42A0-98FD-FA6043A8FE8A}"/>
+  <xr:revisionPtr revIDLastSave="88" documentId="8_{BF3B047A-36C0-4AD4-A0BA-7FD3D60567F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1A847FAC-FF5C-4556-BAE0-746F90154346}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{03E7A685-4EE0-4A4E-B4B4-B1F660F8462C}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{03E7A685-4EE0-4A4E-B4B4-B1F660F8462C}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="172" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="240" uniqueCount="31">
   <si>
     <t>Week</t>
   </si>
@@ -121,6 +121,15 @@
   </si>
   <si>
     <t>January 5–9, 2026</t>
+  </si>
+  <si>
+    <t>Western Delta</t>
+  </si>
+  <si>
+    <t>January 12–16, 2026</t>
+  </si>
+  <si>
+    <t>January 19–23, 2026</t>
   </si>
 </sst>
 </file>
@@ -168,7 +177,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -182,6 +191,15 @@
     </xf>
     <xf numFmtId="3" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -517,7 +535,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{91E6CDBE-81F8-437E-8236-059C4BBF9395}">
-  <dimension ref="A1:K49"/>
+  <dimension ref="A1:K67"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="19.85546875" bestFit="1" customWidth="1"/>
@@ -2239,6 +2257,636 @@
         <v>26236</v>
       </c>
     </row>
+    <row r="50" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A50" s="4">
+        <v>7</v>
+      </c>
+      <c r="B50" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="C50" s="4">
+        <v>3</v>
+      </c>
+      <c r="D50" s="4">
+        <v>12</v>
+      </c>
+      <c r="E50" s="4">
+        <v>0</v>
+      </c>
+      <c r="F50" s="4">
+        <v>0</v>
+      </c>
+      <c r="G50" s="4">
+        <v>0</v>
+      </c>
+      <c r="H50" s="5">
+        <v>53249</v>
+      </c>
+      <c r="I50" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="J50" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="K50" s="4" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="51" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A51" s="4">
+        <v>7</v>
+      </c>
+      <c r="B51" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="C51" s="4">
+        <v>0</v>
+      </c>
+      <c r="D51" s="4">
+        <v>0</v>
+      </c>
+      <c r="E51" s="4">
+        <v>0</v>
+      </c>
+      <c r="F51" s="4">
+        <v>0</v>
+      </c>
+      <c r="G51" s="4">
+        <v>0</v>
+      </c>
+      <c r="H51" s="4">
+        <v>0</v>
+      </c>
+      <c r="I51" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="J51" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="K51" s="4" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="52" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A52" s="4">
+        <v>7</v>
+      </c>
+      <c r="B52" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="C52" s="4">
+        <v>0</v>
+      </c>
+      <c r="D52" s="4">
+        <v>0</v>
+      </c>
+      <c r="E52" s="4">
+        <v>0</v>
+      </c>
+      <c r="F52" s="4">
+        <v>0</v>
+      </c>
+      <c r="G52" s="4">
+        <v>0</v>
+      </c>
+      <c r="H52" s="4">
+        <v>0</v>
+      </c>
+      <c r="I52" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="J52" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="K52" s="4" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="53" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A53" s="4">
+        <v>7</v>
+      </c>
+      <c r="B53" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="C53" s="4">
+        <v>3</v>
+      </c>
+      <c r="D53" s="4">
+        <v>12</v>
+      </c>
+      <c r="E53" s="4">
+        <v>0</v>
+      </c>
+      <c r="F53" s="4">
+        <v>0</v>
+      </c>
+      <c r="G53" s="4">
+        <v>0</v>
+      </c>
+      <c r="H53" s="5">
+        <v>43072</v>
+      </c>
+      <c r="I53" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="J53" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="K53" s="4" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="54" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A54" s="4">
+        <v>7</v>
+      </c>
+      <c r="B54" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="C54" s="4">
+        <v>0</v>
+      </c>
+      <c r="D54" s="4">
+        <v>0</v>
+      </c>
+      <c r="E54" s="4">
+        <v>0</v>
+      </c>
+      <c r="F54" s="4">
+        <v>0</v>
+      </c>
+      <c r="G54" s="4">
+        <v>0</v>
+      </c>
+      <c r="H54" s="4">
+        <v>0</v>
+      </c>
+      <c r="I54" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="J54" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="K54" s="4" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="55" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A55" s="4">
+        <v>7</v>
+      </c>
+      <c r="B55" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="C55" s="4">
+        <v>0</v>
+      </c>
+      <c r="D55" s="4">
+        <v>0</v>
+      </c>
+      <c r="E55" s="4">
+        <v>0</v>
+      </c>
+      <c r="F55" s="4">
+        <v>0</v>
+      </c>
+      <c r="G55" s="4">
+        <v>0</v>
+      </c>
+      <c r="H55" s="4">
+        <v>0</v>
+      </c>
+      <c r="I55" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="J55" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="K55" s="4" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="56" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A56" s="4">
+        <v>7</v>
+      </c>
+      <c r="B56" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="C56" s="4">
+        <v>0</v>
+      </c>
+      <c r="D56" s="4">
+        <v>0</v>
+      </c>
+      <c r="E56" s="4">
+        <v>0</v>
+      </c>
+      <c r="F56" s="4">
+        <v>0</v>
+      </c>
+      <c r="G56" s="4">
+        <v>0</v>
+      </c>
+      <c r="H56" s="4">
+        <v>0</v>
+      </c>
+      <c r="I56" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="J56" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="K56" s="4" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="57" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A57" s="4">
+        <v>7</v>
+      </c>
+      <c r="B57" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="C57" s="4">
+        <v>3</v>
+      </c>
+      <c r="D57" s="4">
+        <v>12</v>
+      </c>
+      <c r="E57" s="4">
+        <v>0</v>
+      </c>
+      <c r="F57" s="4">
+        <v>0</v>
+      </c>
+      <c r="G57" s="4">
+        <v>0</v>
+      </c>
+      <c r="H57" s="5">
+        <v>41695</v>
+      </c>
+      <c r="I57" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="J57" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="K57" s="4" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="58" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A58" s="4">
+        <v>7</v>
+      </c>
+      <c r="B58" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="C58" s="4">
+        <v>9</v>
+      </c>
+      <c r="D58" s="4">
+        <v>36</v>
+      </c>
+      <c r="E58" s="4">
+        <v>0</v>
+      </c>
+      <c r="F58" s="4">
+        <v>0</v>
+      </c>
+      <c r="G58" s="4">
+        <v>0</v>
+      </c>
+      <c r="H58" s="5">
+        <v>138016</v>
+      </c>
+      <c r="I58" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="J58" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="K58" s="4" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="59" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A59" s="4">
+        <v>8</v>
+      </c>
+      <c r="B59" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="C59" s="4">
+        <v>3</v>
+      </c>
+      <c r="D59" s="4">
+        <v>12</v>
+      </c>
+      <c r="E59" s="4">
+        <v>0</v>
+      </c>
+      <c r="F59" s="4">
+        <v>0</v>
+      </c>
+      <c r="G59" s="4">
+        <v>0</v>
+      </c>
+      <c r="H59" s="5">
+        <v>59695</v>
+      </c>
+      <c r="I59" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="J59" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="K59" s="4" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="60" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A60" s="4">
+        <v>8</v>
+      </c>
+      <c r="B60" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="C60" s="4">
+        <v>3</v>
+      </c>
+      <c r="D60" s="4">
+        <v>12</v>
+      </c>
+      <c r="E60" s="4">
+        <v>0</v>
+      </c>
+      <c r="F60" s="4">
+        <v>0</v>
+      </c>
+      <c r="G60" s="4">
+        <v>0</v>
+      </c>
+      <c r="H60" s="5">
+        <v>48484</v>
+      </c>
+      <c r="I60" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="J60" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="K60" s="4" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="61" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A61" s="4">
+        <v>8</v>
+      </c>
+      <c r="B61" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="C61" s="4">
+        <v>0</v>
+      </c>
+      <c r="D61" s="4">
+        <v>0</v>
+      </c>
+      <c r="E61" s="4">
+        <v>0</v>
+      </c>
+      <c r="F61" s="4">
+        <v>0</v>
+      </c>
+      <c r="G61" s="4">
+        <v>0</v>
+      </c>
+      <c r="H61" s="4">
+        <v>0</v>
+      </c>
+      <c r="I61" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="J61" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="K61" s="4" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="62" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A62" s="4">
+        <v>8</v>
+      </c>
+      <c r="B62" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="C62" s="4">
+        <v>3</v>
+      </c>
+      <c r="D62" s="4">
+        <v>12</v>
+      </c>
+      <c r="E62" s="4">
+        <v>0</v>
+      </c>
+      <c r="F62" s="4">
+        <v>0</v>
+      </c>
+      <c r="G62" s="4">
+        <v>0</v>
+      </c>
+      <c r="H62" s="5">
+        <v>52223</v>
+      </c>
+      <c r="I62" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="J62" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="K62" s="4" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="63" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A63" s="4">
+        <v>8</v>
+      </c>
+      <c r="B63" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="C63" s="4">
+        <v>0</v>
+      </c>
+      <c r="D63" s="4">
+        <v>0</v>
+      </c>
+      <c r="E63" s="4">
+        <v>0</v>
+      </c>
+      <c r="F63" s="4">
+        <v>0</v>
+      </c>
+      <c r="G63" s="4">
+        <v>0</v>
+      </c>
+      <c r="H63" s="4">
+        <v>0</v>
+      </c>
+      <c r="I63" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="J63" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="K63" s="4" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="64" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A64" s="4">
+        <v>8</v>
+      </c>
+      <c r="B64" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="C64" s="4">
+        <v>3</v>
+      </c>
+      <c r="D64" s="4">
+        <v>10</v>
+      </c>
+      <c r="E64" s="4">
+        <v>1</v>
+      </c>
+      <c r="F64" s="4">
+        <v>0</v>
+      </c>
+      <c r="G64" s="4">
+        <v>0</v>
+      </c>
+      <c r="H64" s="5">
+        <v>34478</v>
+      </c>
+      <c r="I64" s="4">
+        <v>258</v>
+      </c>
+      <c r="J64" s="4">
+        <v>16</v>
+      </c>
+      <c r="K64" s="5">
+        <v>1219</v>
+      </c>
+    </row>
+    <row r="65" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A65" s="4">
+        <v>8</v>
+      </c>
+      <c r="B65" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="C65" s="4">
+        <v>6</v>
+      </c>
+      <c r="D65" s="4">
+        <v>24</v>
+      </c>
+      <c r="E65" s="4">
+        <v>0</v>
+      </c>
+      <c r="F65" s="4">
+        <v>0</v>
+      </c>
+      <c r="G65" s="4">
+        <v>0</v>
+      </c>
+      <c r="H65" s="5">
+        <v>81962</v>
+      </c>
+      <c r="I65" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="J65" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="K65" s="4" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="66" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A66" s="4">
+        <v>8</v>
+      </c>
+      <c r="B66" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="C66" s="4">
+        <v>3</v>
+      </c>
+      <c r="D66" s="4">
+        <v>10</v>
+      </c>
+      <c r="E66" s="4">
+        <v>0</v>
+      </c>
+      <c r="F66" s="4">
+        <v>0</v>
+      </c>
+      <c r="G66" s="4">
+        <v>0</v>
+      </c>
+      <c r="H66" s="5">
+        <v>30268</v>
+      </c>
+      <c r="I66" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="J66" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="K66" s="4" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="67" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A67" s="4">
+        <v>8</v>
+      </c>
+      <c r="B67" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="C67" s="4">
+        <v>21</v>
+      </c>
+      <c r="D67" s="4">
+        <v>80</v>
+      </c>
+      <c r="E67" s="4">
+        <v>1</v>
+      </c>
+      <c r="F67" s="4">
+        <v>0</v>
+      </c>
+      <c r="G67" s="4">
+        <v>0</v>
+      </c>
+      <c r="H67" s="5">
+        <v>307111</v>
+      </c>
+      <c r="I67" s="4">
+        <v>258</v>
+      </c>
+      <c r="J67" s="4">
+        <v>16</v>
+      </c>
+      <c r="K67" s="5">
+        <v>1219</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
@@ -2247,7 +2895,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DC5A6928-3806-4082-94AB-A52936AB7317}">
-  <dimension ref="A1:B7"/>
+  <dimension ref="A1:B9"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5.7109375" bestFit="1" customWidth="1"/>
@@ -2255,59 +2903,75 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
+      <c r="A1" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="6" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A2">
+      <c r="A2" s="6">
         <v>1</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="6" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A3">
+      <c r="A3" s="6">
         <v>2</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" s="6" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A4">
-        <v>3</v>
-      </c>
-      <c r="B4" t="s">
+      <c r="A4" s="6">
+        <v>3</v>
+      </c>
+      <c r="B4" s="6" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A5">
+      <c r="A5" s="6">
         <v>4</v>
       </c>
-      <c r="B5" t="s">
+      <c r="B5" s="6" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A6">
+      <c r="A6" s="6">
         <v>5</v>
       </c>
-      <c r="B6" t="s">
+      <c r="B6" s="6" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A7" s="4">
+      <c r="A7" s="7">
         <v>6</v>
       </c>
-      <c r="B7" s="4" t="s">
+      <c r="B7" s="7" t="s">
         <v>27</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A8" s="7">
+        <v>7</v>
+      </c>
+      <c r="B8" s="8" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A9" s="7">
+        <v>8</v>
+      </c>
+      <c r="B9" s="8" t="s">
+        <v>30</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Code updates for alt fig text, typos
</commit_message>
<xml_diff>
--- a/data_raw/smelt/abundance_estimates.xlsx
+++ b/data_raw/smelt/abundance_estimates.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://doimspp-my.sharepoint.com/personal/geasterbrook_usbr_gov/Documents/My Projects/SMT/Assessment/samt_smt_assessments/data_raw/smelt/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://doimspp-my.sharepoint.com/personal/lmccormick_usbr_gov/Documents/Documents/Research/R/samt_smt_assessments/data_raw/smelt/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="79" documentId="8_{BF3B047A-36C0-4AD4-A0BA-7FD3D60567F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{97FD1B19-9E17-42A0-98FD-FA6043A8FE8A}"/>
+  <xr:revisionPtr revIDLastSave="85" documentId="8_{BF3B047A-36C0-4AD4-A0BA-7FD3D60567F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F95B8350-1224-4344-9D96-47EE1447852A}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{03E7A685-4EE0-4A4E-B4B4-B1F660F8462C}"/>
+    <workbookView xWindow="12936" yWindow="-14880" windowWidth="18132" windowHeight="12984" activeTab="1" xr2:uid="{03E7A685-4EE0-4A4E-B4B4-B1F660F8462C}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="172" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="209" uniqueCount="30">
   <si>
     <t>Week</t>
   </si>
@@ -121,13 +121,19 @@
   </si>
   <si>
     <t>January 5–9, 2026</t>
+  </si>
+  <si>
+    <t>Western Delta</t>
+  </si>
+  <si>
+    <t>January 12–16, 2026</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -135,25 +141,13 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF000000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFFF"/>
-        <bgColor indexed="64"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -168,21 +162,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="3" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -517,14 +499,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{91E6CDBE-81F8-437E-8236-059C4BBF9395}">
-  <dimension ref="A1:K49"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:K58"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="19.85546875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="16.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="19.88671875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="16.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -559,7 +541,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>1</v>
       </c>
@@ -594,7 +576,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>1</v>
       </c>
@@ -629,7 +611,7 @@
         <v>10740</v>
       </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>1</v>
       </c>
@@ -664,7 +646,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>1</v>
       </c>
@@ -699,7 +681,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>1</v>
       </c>
@@ -734,7 +716,7 @@
         <v>3065</v>
       </c>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>1</v>
       </c>
@@ -769,7 +751,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>1</v>
       </c>
@@ -804,7 +786,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>1</v>
       </c>
@@ -839,7 +821,7 @@
         <v>12103</v>
       </c>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>2</v>
       </c>
@@ -874,7 +856,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>2</v>
       </c>
@@ -909,7 +891,7 @@
         <v>29101</v>
       </c>
     </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A12">
         <v>2</v>
       </c>
@@ -944,7 +926,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>2</v>
       </c>
@@ -979,7 +961,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A14">
         <v>2</v>
       </c>
@@ -1014,7 +996,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A15">
         <v>2</v>
       </c>
@@ -1049,7 +1031,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A16">
         <v>2</v>
       </c>
@@ -1084,7 +1066,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A17">
         <v>2</v>
       </c>
@@ -1119,7 +1101,7 @@
         <v>29101</v>
       </c>
     </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A18">
         <v>3</v>
       </c>
@@ -1154,7 +1136,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A19">
         <v>3</v>
       </c>
@@ -1189,7 +1171,7 @@
         <v>8836</v>
       </c>
     </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A20">
         <v>3</v>
       </c>
@@ -1224,7 +1206,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A21">
         <v>3</v>
       </c>
@@ -1259,7 +1241,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A22">
         <v>3</v>
       </c>
@@ -1294,7 +1276,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A23">
         <v>3</v>
       </c>
@@ -1329,7 +1311,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A24">
         <v>3</v>
       </c>
@@ -1364,7 +1346,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A25">
         <v>3</v>
       </c>
@@ -1399,7 +1381,7 @@
         <v>8836</v>
       </c>
     </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A26">
         <v>4</v>
       </c>
@@ -1434,7 +1416,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A27">
         <v>4</v>
       </c>
@@ -1469,7 +1451,7 @@
         <v>11902</v>
       </c>
     </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A28">
         <v>4</v>
       </c>
@@ -1504,7 +1486,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="29" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A29">
         <v>4</v>
       </c>
@@ -1539,7 +1521,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="30" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A30">
         <v>4</v>
       </c>
@@ -1574,7 +1556,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="31" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A31">
         <v>4</v>
       </c>
@@ -1609,7 +1591,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="32" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A32">
         <v>4</v>
       </c>
@@ -1644,7 +1626,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="33" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A33">
         <v>4</v>
       </c>
@@ -1679,7 +1661,7 @@
         <v>11902</v>
       </c>
     </row>
-    <row r="34" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A34">
         <v>5</v>
       </c>
@@ -1714,7 +1696,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="35" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A35">
         <v>5</v>
       </c>
@@ -1749,7 +1731,7 @@
         <v>20185</v>
       </c>
     </row>
-    <row r="36" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A36">
         <v>5</v>
       </c>
@@ -1784,7 +1766,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="37" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A37">
         <v>5</v>
       </c>
@@ -1819,7 +1801,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="38" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A38">
         <v>5</v>
       </c>
@@ -1854,7 +1836,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="39" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A39">
         <v>5</v>
       </c>
@@ -1889,7 +1871,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="40" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A40">
         <v>5</v>
       </c>
@@ -1924,319 +1906,634 @@
         <v>13</v>
       </c>
     </row>
-    <row r="41" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A41" s="2">
+    <row r="41" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A41">
         <v>5</v>
       </c>
-      <c r="B41" s="2" t="s">
+      <c r="B41" t="s">
         <v>19</v>
       </c>
-      <c r="C41" s="2">
+      <c r="C41">
         <v>28</v>
       </c>
-      <c r="D41" s="2">
+      <c r="D41">
         <v>105</v>
       </c>
-      <c r="E41" s="2">
+      <c r="E41">
         <v>5</v>
       </c>
-      <c r="F41" s="2">
-        <v>0</v>
-      </c>
-      <c r="G41" s="2">
-        <v>0</v>
-      </c>
-      <c r="H41" s="3">
+      <c r="F41">
+        <v>0</v>
+      </c>
+      <c r="G41">
+        <v>0</v>
+      </c>
+      <c r="H41">
         <v>382087</v>
       </c>
-      <c r="I41" s="3">
+      <c r="I41">
         <v>6821</v>
       </c>
-      <c r="J41" s="3">
+      <c r="J41">
         <v>1477</v>
       </c>
-      <c r="K41" s="3">
+      <c r="K41">
         <v>20185</v>
       </c>
     </row>
-    <row r="42" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A42" s="4">
-        <v>6</v>
-      </c>
-      <c r="B42" s="4" t="s">
+    <row r="42" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A42">
+        <v>6</v>
+      </c>
+      <c r="B42" t="s">
         <v>11</v>
       </c>
-      <c r="C42" s="4">
-        <v>6</v>
-      </c>
-      <c r="D42" s="4">
+      <c r="C42">
+        <v>6</v>
+      </c>
+      <c r="D42">
         <v>22</v>
       </c>
-      <c r="E42" s="4">
-        <v>0</v>
-      </c>
-      <c r="F42" s="4">
-        <v>0</v>
-      </c>
-      <c r="G42" s="4">
-        <v>0</v>
-      </c>
-      <c r="H42" s="5">
+      <c r="E42">
+        <v>0</v>
+      </c>
+      <c r="F42">
+        <v>0</v>
+      </c>
+      <c r="G42">
+        <v>0</v>
+      </c>
+      <c r="H42">
         <v>85390</v>
       </c>
-      <c r="I42" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="J42" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="K42" s="4" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="43" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A43" s="4">
-        <v>6</v>
-      </c>
-      <c r="B43" s="4" t="s">
+      <c r="I42" t="s">
+        <v>12</v>
+      </c>
+      <c r="J42" t="s">
+        <v>13</v>
+      </c>
+      <c r="K42" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="43" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A43">
+        <v>6</v>
+      </c>
+      <c r="B43" t="s">
         <v>14</v>
       </c>
-      <c r="C43" s="4">
-        <v>6</v>
-      </c>
-      <c r="D43" s="4">
+      <c r="C43">
+        <v>6</v>
+      </c>
+      <c r="D43">
         <v>16</v>
       </c>
-      <c r="E43" s="4">
-        <v>6</v>
-      </c>
-      <c r="F43" s="4">
-        <v>0</v>
-      </c>
-      <c r="G43" s="4">
-        <v>0</v>
-      </c>
-      <c r="H43" s="5">
+      <c r="E43">
+        <v>6</v>
+      </c>
+      <c r="F43">
+        <v>0</v>
+      </c>
+      <c r="G43">
+        <v>0</v>
+      </c>
+      <c r="H43">
         <v>61809</v>
       </c>
-      <c r="I43" s="5">
+      <c r="I43">
         <v>8963</v>
       </c>
-      <c r="J43" s="5">
+      <c r="J43">
         <v>1984</v>
       </c>
-      <c r="K43" s="5">
+      <c r="K43">
         <v>26236</v>
       </c>
     </row>
-    <row r="44" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A44" s="4">
-        <v>6</v>
-      </c>
-      <c r="B44" s="4" t="s">
+    <row r="44" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A44">
+        <v>6</v>
+      </c>
+      <c r="B44" t="s">
         <v>15</v>
       </c>
-      <c r="C44" s="4">
-        <v>6</v>
-      </c>
-      <c r="D44" s="4">
+      <c r="C44">
+        <v>6</v>
+      </c>
+      <c r="D44">
         <v>22</v>
       </c>
-      <c r="E44" s="4">
-        <v>0</v>
-      </c>
-      <c r="F44" s="4">
-        <v>0</v>
-      </c>
-      <c r="G44" s="4">
-        <v>0</v>
-      </c>
-      <c r="H44" s="5">
+      <c r="E44">
+        <v>0</v>
+      </c>
+      <c r="F44">
+        <v>0</v>
+      </c>
+      <c r="G44">
+        <v>0</v>
+      </c>
+      <c r="H44">
         <v>88609</v>
       </c>
-      <c r="I44" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="J44" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="K44" s="4" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="45" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A45" s="4">
-        <v>6</v>
-      </c>
-      <c r="B45" s="4" t="s">
+      <c r="I44" t="s">
+        <v>12</v>
+      </c>
+      <c r="J44" t="s">
+        <v>13</v>
+      </c>
+      <c r="K44" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="45" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A45">
+        <v>6</v>
+      </c>
+      <c r="B45" t="s">
         <v>16</v>
       </c>
-      <c r="C45" s="4">
+      <c r="C45">
         <v>2</v>
       </c>
-      <c r="D45" s="4">
+      <c r="D45">
         <v>8</v>
       </c>
-      <c r="E45" s="4">
-        <v>0</v>
-      </c>
-      <c r="F45" s="4">
-        <v>0</v>
-      </c>
-      <c r="G45" s="4">
-        <v>0</v>
-      </c>
-      <c r="H45" s="5">
+      <c r="E45">
+        <v>0</v>
+      </c>
+      <c r="F45">
+        <v>0</v>
+      </c>
+      <c r="G45">
+        <v>0</v>
+      </c>
+      <c r="H45">
         <v>24368</v>
       </c>
-      <c r="I45" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="J45" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="K45" s="4" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="46" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A46" s="4">
-        <v>6</v>
-      </c>
-      <c r="B46" s="4" t="s">
+      <c r="I45" t="s">
+        <v>12</v>
+      </c>
+      <c r="J45" t="s">
+        <v>13</v>
+      </c>
+      <c r="K45" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="46" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A46">
+        <v>6</v>
+      </c>
+      <c r="B46" t="s">
         <v>17</v>
       </c>
-      <c r="C46" s="4">
-        <v>3</v>
-      </c>
-      <c r="D46" s="4">
-        <v>12</v>
-      </c>
-      <c r="E46" s="4">
-        <v>0</v>
-      </c>
-      <c r="F46" s="4">
-        <v>0</v>
-      </c>
-      <c r="G46" s="4">
-        <v>0</v>
-      </c>
-      <c r="H46" s="5">
+      <c r="C46">
+        <v>3</v>
+      </c>
+      <c r="D46">
+        <v>12</v>
+      </c>
+      <c r="E46">
+        <v>0</v>
+      </c>
+      <c r="F46">
+        <v>0</v>
+      </c>
+      <c r="G46">
+        <v>0</v>
+      </c>
+      <c r="H46">
         <v>42440</v>
       </c>
-      <c r="I46" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="J46" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="K46" s="4" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="47" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A47" s="4">
-        <v>6</v>
-      </c>
-      <c r="B47" s="4" t="s">
+      <c r="I46" t="s">
+        <v>12</v>
+      </c>
+      <c r="J46" t="s">
+        <v>13</v>
+      </c>
+      <c r="K46" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="47" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A47">
+        <v>6</v>
+      </c>
+      <c r="B47" t="s">
         <v>18</v>
       </c>
-      <c r="C47" s="4">
-        <v>6</v>
-      </c>
-      <c r="D47" s="4">
+      <c r="C47">
+        <v>6</v>
+      </c>
+      <c r="D47">
         <v>24</v>
       </c>
-      <c r="E47" s="4">
-        <v>0</v>
-      </c>
-      <c r="F47" s="4">
-        <v>0</v>
-      </c>
-      <c r="G47" s="4">
-        <v>0</v>
-      </c>
-      <c r="H47" s="5">
+      <c r="E47">
+        <v>0</v>
+      </c>
+      <c r="F47">
+        <v>0</v>
+      </c>
+      <c r="G47">
+        <v>0</v>
+      </c>
+      <c r="H47">
         <v>89192</v>
       </c>
-      <c r="I47" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="J47" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="K47" s="4" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="48" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A48" s="4">
-        <v>6</v>
-      </c>
-      <c r="B48" s="4" t="s">
+      <c r="I47" t="s">
+        <v>12</v>
+      </c>
+      <c r="J47" t="s">
+        <v>13</v>
+      </c>
+      <c r="K47" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="48" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A48">
+        <v>6</v>
+      </c>
+      <c r="B48" t="s">
         <v>22</v>
       </c>
-      <c r="C48" s="4">
+      <c r="C48">
         <v>5</v>
       </c>
-      <c r="D48" s="4">
+      <c r="D48">
         <v>20</v>
       </c>
-      <c r="E48" s="4">
-        <v>0</v>
-      </c>
-      <c r="F48" s="4">
-        <v>0</v>
-      </c>
-      <c r="G48" s="4">
-        <v>0</v>
-      </c>
-      <c r="H48" s="5">
+      <c r="E48">
+        <v>0</v>
+      </c>
+      <c r="F48">
+        <v>0</v>
+      </c>
+      <c r="G48">
+        <v>0</v>
+      </c>
+      <c r="H48">
         <v>78554</v>
       </c>
-      <c r="I48" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="J48" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="K48" s="4" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="49" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A49" s="4">
-        <v>6</v>
-      </c>
-      <c r="B49" s="4" t="s">
+      <c r="I48" t="s">
+        <v>12</v>
+      </c>
+      <c r="J48" t="s">
+        <v>13</v>
+      </c>
+      <c r="K48" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="49" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A49">
+        <v>6</v>
+      </c>
+      <c r="B49" t="s">
         <v>19</v>
       </c>
-      <c r="C49" s="4">
+      <c r="C49">
         <v>34</v>
       </c>
-      <c r="D49" s="4">
+      <c r="D49">
         <v>124</v>
       </c>
-      <c r="E49" s="4">
-        <v>6</v>
-      </c>
-      <c r="F49" s="4">
-        <v>0</v>
-      </c>
-      <c r="G49" s="4">
-        <v>0</v>
-      </c>
-      <c r="H49" s="5">
+      <c r="E49">
+        <v>6</v>
+      </c>
+      <c r="F49">
+        <v>0</v>
+      </c>
+      <c r="G49">
+        <v>0</v>
+      </c>
+      <c r="H49">
         <v>470362</v>
       </c>
-      <c r="I49" s="5">
+      <c r="I49">
         <v>8963</v>
       </c>
-      <c r="J49" s="5">
+      <c r="J49">
         <v>1984</v>
       </c>
-      <c r="K49" s="5">
+      <c r="K49">
         <v>26236</v>
+      </c>
+    </row>
+    <row r="50" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A50">
+        <v>7</v>
+      </c>
+      <c r="B50" t="s">
+        <v>28</v>
+      </c>
+      <c r="C50">
+        <v>3</v>
+      </c>
+      <c r="D50">
+        <v>12</v>
+      </c>
+      <c r="E50">
+        <v>0</v>
+      </c>
+      <c r="F50">
+        <v>0</v>
+      </c>
+      <c r="G50">
+        <v>0</v>
+      </c>
+      <c r="H50" s="1">
+        <v>53249</v>
+      </c>
+      <c r="I50" t="s">
+        <v>12</v>
+      </c>
+      <c r="J50" t="s">
+        <v>13</v>
+      </c>
+      <c r="K50" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="51" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A51">
+        <v>7</v>
+      </c>
+      <c r="B51" t="s">
+        <v>11</v>
+      </c>
+      <c r="C51">
+        <v>0</v>
+      </c>
+      <c r="D51">
+        <v>0</v>
+      </c>
+      <c r="E51">
+        <v>0</v>
+      </c>
+      <c r="F51">
+        <v>0</v>
+      </c>
+      <c r="G51">
+        <v>0</v>
+      </c>
+      <c r="H51">
+        <v>0</v>
+      </c>
+      <c r="I51" t="s">
+        <v>13</v>
+      </c>
+      <c r="J51" t="s">
+        <v>13</v>
+      </c>
+      <c r="K51" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="52" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A52">
+        <v>7</v>
+      </c>
+      <c r="B52" t="s">
+        <v>14</v>
+      </c>
+      <c r="C52">
+        <v>0</v>
+      </c>
+      <c r="D52">
+        <v>0</v>
+      </c>
+      <c r="E52">
+        <v>0</v>
+      </c>
+      <c r="F52">
+        <v>0</v>
+      </c>
+      <c r="G52">
+        <v>0</v>
+      </c>
+      <c r="H52">
+        <v>0</v>
+      </c>
+      <c r="I52" t="s">
+        <v>13</v>
+      </c>
+      <c r="J52" t="s">
+        <v>13</v>
+      </c>
+      <c r="K52" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="53" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A53">
+        <v>7</v>
+      </c>
+      <c r="B53" t="s">
+        <v>15</v>
+      </c>
+      <c r="C53">
+        <v>3</v>
+      </c>
+      <c r="D53">
+        <v>12</v>
+      </c>
+      <c r="E53">
+        <v>0</v>
+      </c>
+      <c r="F53">
+        <v>0</v>
+      </c>
+      <c r="G53">
+        <v>0</v>
+      </c>
+      <c r="H53" s="1">
+        <v>43072</v>
+      </c>
+      <c r="I53" t="s">
+        <v>12</v>
+      </c>
+      <c r="J53" t="s">
+        <v>13</v>
+      </c>
+      <c r="K53" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="54" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A54">
+        <v>7</v>
+      </c>
+      <c r="B54" t="s">
+        <v>16</v>
+      </c>
+      <c r="C54">
+        <v>0</v>
+      </c>
+      <c r="D54">
+        <v>0</v>
+      </c>
+      <c r="E54">
+        <v>0</v>
+      </c>
+      <c r="F54">
+        <v>0</v>
+      </c>
+      <c r="G54">
+        <v>0</v>
+      </c>
+      <c r="H54">
+        <v>0</v>
+      </c>
+      <c r="I54" t="s">
+        <v>13</v>
+      </c>
+      <c r="J54" t="s">
+        <v>13</v>
+      </c>
+      <c r="K54" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="55" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A55">
+        <v>7</v>
+      </c>
+      <c r="B55" t="s">
+        <v>17</v>
+      </c>
+      <c r="C55">
+        <v>0</v>
+      </c>
+      <c r="D55">
+        <v>0</v>
+      </c>
+      <c r="E55">
+        <v>0</v>
+      </c>
+      <c r="F55">
+        <v>0</v>
+      </c>
+      <c r="G55">
+        <v>0</v>
+      </c>
+      <c r="H55">
+        <v>0</v>
+      </c>
+      <c r="I55" t="s">
+        <v>13</v>
+      </c>
+      <c r="J55" t="s">
+        <v>13</v>
+      </c>
+      <c r="K55" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="56" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A56">
+        <v>7</v>
+      </c>
+      <c r="B56" t="s">
+        <v>18</v>
+      </c>
+      <c r="C56">
+        <v>0</v>
+      </c>
+      <c r="D56">
+        <v>0</v>
+      </c>
+      <c r="E56">
+        <v>0</v>
+      </c>
+      <c r="F56">
+        <v>0</v>
+      </c>
+      <c r="G56">
+        <v>0</v>
+      </c>
+      <c r="H56">
+        <v>0</v>
+      </c>
+      <c r="I56" t="s">
+        <v>13</v>
+      </c>
+      <c r="J56" t="s">
+        <v>13</v>
+      </c>
+      <c r="K56" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="57" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A57">
+        <v>7</v>
+      </c>
+      <c r="B57" t="s">
+        <v>22</v>
+      </c>
+      <c r="C57">
+        <v>3</v>
+      </c>
+      <c r="D57">
+        <v>12</v>
+      </c>
+      <c r="E57">
+        <v>0</v>
+      </c>
+      <c r="F57">
+        <v>0</v>
+      </c>
+      <c r="G57">
+        <v>0</v>
+      </c>
+      <c r="H57" s="1">
+        <v>41695</v>
+      </c>
+      <c r="I57" t="s">
+        <v>12</v>
+      </c>
+      <c r="J57" t="s">
+        <v>13</v>
+      </c>
+      <c r="K57" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="58" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A58">
+        <v>7</v>
+      </c>
+      <c r="B58" t="s">
+        <v>19</v>
+      </c>
+      <c r="C58">
+        <v>9</v>
+      </c>
+      <c r="D58">
+        <v>36</v>
+      </c>
+      <c r="E58">
+        <v>0</v>
+      </c>
+      <c r="F58">
+        <v>0</v>
+      </c>
+      <c r="G58">
+        <v>0</v>
+      </c>
+      <c r="H58" s="1">
+        <v>138016</v>
+      </c>
+      <c r="I58" t="s">
+        <v>12</v>
+      </c>
+      <c r="J58" t="s">
+        <v>13</v>
+      </c>
+      <c r="K58" t="s">
+        <v>13</v>
       </c>
     </row>
   </sheetData>
@@ -2247,14 +2544,14 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DC5A6928-3806-4082-94AB-A52936AB7317}">
-  <dimension ref="A1:B7"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:B8"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="27.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="5.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="27.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -2262,7 +2559,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>1</v>
       </c>
@@ -2270,7 +2567,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>2</v>
       </c>
@@ -2278,7 +2575,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>3</v>
       </c>
@@ -2286,7 +2583,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>4</v>
       </c>
@@ -2294,7 +2591,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>5</v>
       </c>
@@ -2302,12 +2599,20 @@
         <v>26</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A7" s="4">
-        <v>6</v>
-      </c>
-      <c r="B7" s="4" t="s">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A7">
+        <v>6</v>
+      </c>
+      <c r="B7" t="s">
         <v>27</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A8">
+        <v>7</v>
+      </c>
+      <c r="B8" t="s">
+        <v>29</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Smelt assessment updates 2/2
</commit_message>
<xml_diff>
--- a/data_raw/smelt/abundance_estimates.xlsx
+++ b/data_raw/smelt/abundance_estimates.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://doimspp-my.sharepoint.com/personal/geasterbrook_usbr_gov/Documents/My Projects/SMT/Assessment/samt_smt_assessments/data_raw/smelt/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://doimspp-my.sharepoint.com/personal/lmccormick_usbr_gov/Documents/Documents/Research/R/samt_smt_assessments/data_raw/smelt/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="88" documentId="8_{BF3B047A-36C0-4AD4-A0BA-7FD3D60567F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1A847FAC-FF5C-4556-BAE0-746F90154346}"/>
+  <xr:revisionPtr revIDLastSave="94" documentId="8_{BF3B047A-36C0-4AD4-A0BA-7FD3D60567F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9C55109B-7597-4BD3-8F81-E592B50DADC1}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-45" windowWidth="29040" windowHeight="15720" xr2:uid="{03E7A685-4EE0-4A4E-B4B4-B1F660F8462C}"/>
+    <workbookView xWindow="13680" yWindow="-14328" windowWidth="19584" windowHeight="11040" xr2:uid="{03E7A685-4EE0-4A4E-B4B4-B1F660F8462C}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="240" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="271" uniqueCount="32">
   <si>
     <t>Week</t>
   </si>
@@ -131,12 +131,15 @@
   <si>
     <t>January 19–23, 2026</t>
   </si>
+  <si>
+    <t>January 26–30, 2026</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -144,25 +147,13 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF000000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFFF"/>
-        <bgColor indexed="64"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -177,7 +168,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -186,20 +177,8 @@
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="3" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -535,14 +514,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{91E6CDBE-81F8-437E-8236-059C4BBF9395}">
-  <dimension ref="A1:K67"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:K76"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="19.85546875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="16.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="19.88671875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="16.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -577,7 +556,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>1</v>
       </c>
@@ -612,7 +591,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>1</v>
       </c>
@@ -647,7 +626,7 @@
         <v>10740</v>
       </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>1</v>
       </c>
@@ -682,7 +661,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>1</v>
       </c>
@@ -717,7 +696,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>1</v>
       </c>
@@ -752,7 +731,7 @@
         <v>3065</v>
       </c>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>1</v>
       </c>
@@ -787,7 +766,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>1</v>
       </c>
@@ -822,7 +801,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>1</v>
       </c>
@@ -857,7 +836,7 @@
         <v>12103</v>
       </c>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>2</v>
       </c>
@@ -892,7 +871,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>2</v>
       </c>
@@ -927,7 +906,7 @@
         <v>29101</v>
       </c>
     </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A12">
         <v>2</v>
       </c>
@@ -962,7 +941,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>2</v>
       </c>
@@ -997,7 +976,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A14">
         <v>2</v>
       </c>
@@ -1032,7 +1011,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A15">
         <v>2</v>
       </c>
@@ -1067,7 +1046,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A16">
         <v>2</v>
       </c>
@@ -1102,7 +1081,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A17">
         <v>2</v>
       </c>
@@ -1137,7 +1116,7 @@
         <v>29101</v>
       </c>
     </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A18">
         <v>3</v>
       </c>
@@ -1172,7 +1151,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A19">
         <v>3</v>
       </c>
@@ -1207,7 +1186,7 @@
         <v>8836</v>
       </c>
     </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A20">
         <v>3</v>
       </c>
@@ -1242,7 +1221,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A21">
         <v>3</v>
       </c>
@@ -1277,7 +1256,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A22">
         <v>3</v>
       </c>
@@ -1312,7 +1291,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A23">
         <v>3</v>
       </c>
@@ -1347,7 +1326,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A24">
         <v>3</v>
       </c>
@@ -1382,7 +1361,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A25">
         <v>3</v>
       </c>
@@ -1417,7 +1396,7 @@
         <v>8836</v>
       </c>
     </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A26">
         <v>4</v>
       </c>
@@ -1452,7 +1431,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A27">
         <v>4</v>
       </c>
@@ -1487,7 +1466,7 @@
         <v>11902</v>
       </c>
     </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A28">
         <v>4</v>
       </c>
@@ -1522,7 +1501,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="29" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A29">
         <v>4</v>
       </c>
@@ -1557,7 +1536,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="30" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A30">
         <v>4</v>
       </c>
@@ -1592,7 +1571,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="31" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A31">
         <v>4</v>
       </c>
@@ -1627,7 +1606,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="32" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A32">
         <v>4</v>
       </c>
@@ -1662,7 +1641,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="33" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A33">
         <v>4</v>
       </c>
@@ -1697,7 +1676,7 @@
         <v>11902</v>
       </c>
     </row>
-    <row r="34" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A34">
         <v>5</v>
       </c>
@@ -1732,7 +1711,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="35" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A35">
         <v>5</v>
       </c>
@@ -1767,7 +1746,7 @@
         <v>20185</v>
       </c>
     </row>
-    <row r="36" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A36">
         <v>5</v>
       </c>
@@ -1802,7 +1781,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="37" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A37">
         <v>5</v>
       </c>
@@ -1837,7 +1816,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="38" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A38">
         <v>5</v>
       </c>
@@ -1872,7 +1851,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="39" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A39">
         <v>5</v>
       </c>
@@ -1907,7 +1886,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="40" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A40">
         <v>5</v>
       </c>
@@ -1942,7 +1921,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="41" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A41" s="2">
         <v>5</v>
       </c>
@@ -1977,914 +1956,1229 @@
         <v>20185</v>
       </c>
     </row>
-    <row r="42" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A42" s="4">
+    <row r="42" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A42">
         <v>6</v>
       </c>
-      <c r="B42" s="4" t="s">
+      <c r="B42" t="s">
         <v>11</v>
       </c>
-      <c r="C42" s="4">
+      <c r="C42">
         <v>6</v>
       </c>
-      <c r="D42" s="4">
+      <c r="D42">
         <v>22</v>
       </c>
-      <c r="E42" s="4">
-        <v>0</v>
-      </c>
-      <c r="F42" s="4">
-        <v>0</v>
-      </c>
-      <c r="G42" s="4">
-        <v>0</v>
-      </c>
-      <c r="H42" s="5">
+      <c r="E42">
+        <v>0</v>
+      </c>
+      <c r="F42">
+        <v>0</v>
+      </c>
+      <c r="G42">
+        <v>0</v>
+      </c>
+      <c r="H42">
         <v>85390</v>
       </c>
-      <c r="I42" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="J42" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="K42" s="4" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="43" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A43" s="4">
+      <c r="I42" t="s">
+        <v>12</v>
+      </c>
+      <c r="J42" t="s">
+        <v>13</v>
+      </c>
+      <c r="K42" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="43" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A43">
         <v>6</v>
       </c>
-      <c r="B43" s="4" t="s">
+      <c r="B43" t="s">
         <v>14</v>
       </c>
-      <c r="C43" s="4">
+      <c r="C43">
         <v>6</v>
       </c>
-      <c r="D43" s="4">
+      <c r="D43">
         <v>16</v>
       </c>
-      <c r="E43" s="4">
+      <c r="E43">
         <v>6</v>
       </c>
-      <c r="F43" s="4">
-        <v>0</v>
-      </c>
-      <c r="G43" s="4">
-        <v>0</v>
-      </c>
-      <c r="H43" s="5">
+      <c r="F43">
+        <v>0</v>
+      </c>
+      <c r="G43">
+        <v>0</v>
+      </c>
+      <c r="H43">
         <v>61809</v>
       </c>
-      <c r="I43" s="5">
+      <c r="I43">
         <v>8963</v>
       </c>
-      <c r="J43" s="5">
+      <c r="J43">
         <v>1984</v>
       </c>
-      <c r="K43" s="5">
+      <c r="K43">
         <v>26236</v>
       </c>
     </row>
-    <row r="44" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A44" s="4">
+    <row r="44" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A44">
         <v>6</v>
       </c>
-      <c r="B44" s="4" t="s">
+      <c r="B44" t="s">
         <v>15</v>
       </c>
-      <c r="C44" s="4">
+      <c r="C44">
         <v>6</v>
       </c>
-      <c r="D44" s="4">
+      <c r="D44">
         <v>22</v>
       </c>
-      <c r="E44" s="4">
-        <v>0</v>
-      </c>
-      <c r="F44" s="4">
-        <v>0</v>
-      </c>
-      <c r="G44" s="4">
-        <v>0</v>
-      </c>
-      <c r="H44" s="5">
+      <c r="E44">
+        <v>0</v>
+      </c>
+      <c r="F44">
+        <v>0</v>
+      </c>
+      <c r="G44">
+        <v>0</v>
+      </c>
+      <c r="H44">
         <v>88609</v>
       </c>
-      <c r="I44" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="J44" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="K44" s="4" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="45" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A45" s="4">
+      <c r="I44" t="s">
+        <v>12</v>
+      </c>
+      <c r="J44" t="s">
+        <v>13</v>
+      </c>
+      <c r="K44" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="45" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A45">
         <v>6</v>
       </c>
-      <c r="B45" s="4" t="s">
+      <c r="B45" t="s">
         <v>16</v>
       </c>
-      <c r="C45" s="4">
+      <c r="C45">
         <v>2</v>
       </c>
-      <c r="D45" s="4">
+      <c r="D45">
         <v>8</v>
       </c>
-      <c r="E45" s="4">
-        <v>0</v>
-      </c>
-      <c r="F45" s="4">
-        <v>0</v>
-      </c>
-      <c r="G45" s="4">
-        <v>0</v>
-      </c>
-      <c r="H45" s="5">
+      <c r="E45">
+        <v>0</v>
+      </c>
+      <c r="F45">
+        <v>0</v>
+      </c>
+      <c r="G45">
+        <v>0</v>
+      </c>
+      <c r="H45">
         <v>24368</v>
       </c>
-      <c r="I45" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="J45" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="K45" s="4" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="46" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A46" s="4">
+      <c r="I45" t="s">
+        <v>12</v>
+      </c>
+      <c r="J45" t="s">
+        <v>13</v>
+      </c>
+      <c r="K45" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="46" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A46">
         <v>6</v>
       </c>
-      <c r="B46" s="4" t="s">
+      <c r="B46" t="s">
         <v>17</v>
       </c>
-      <c r="C46" s="4">
-        <v>3</v>
-      </c>
-      <c r="D46" s="4">
-        <v>12</v>
-      </c>
-      <c r="E46" s="4">
-        <v>0</v>
-      </c>
-      <c r="F46" s="4">
-        <v>0</v>
-      </c>
-      <c r="G46" s="4">
-        <v>0</v>
-      </c>
-      <c r="H46" s="5">
+      <c r="C46">
+        <v>3</v>
+      </c>
+      <c r="D46">
+        <v>12</v>
+      </c>
+      <c r="E46">
+        <v>0</v>
+      </c>
+      <c r="F46">
+        <v>0</v>
+      </c>
+      <c r="G46">
+        <v>0</v>
+      </c>
+      <c r="H46">
         <v>42440</v>
       </c>
-      <c r="I46" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="J46" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="K46" s="4" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="47" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A47" s="4">
+      <c r="I46" t="s">
+        <v>12</v>
+      </c>
+      <c r="J46" t="s">
+        <v>13</v>
+      </c>
+      <c r="K46" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="47" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A47">
         <v>6</v>
       </c>
-      <c r="B47" s="4" t="s">
+      <c r="B47" t="s">
         <v>18</v>
       </c>
-      <c r="C47" s="4">
+      <c r="C47">
         <v>6</v>
       </c>
-      <c r="D47" s="4">
+      <c r="D47">
         <v>24</v>
       </c>
-      <c r="E47" s="4">
-        <v>0</v>
-      </c>
-      <c r="F47" s="4">
-        <v>0</v>
-      </c>
-      <c r="G47" s="4">
-        <v>0</v>
-      </c>
-      <c r="H47" s="5">
+      <c r="E47">
+        <v>0</v>
+      </c>
+      <c r="F47">
+        <v>0</v>
+      </c>
+      <c r="G47">
+        <v>0</v>
+      </c>
+      <c r="H47">
         <v>89192</v>
       </c>
-      <c r="I47" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="J47" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="K47" s="4" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="48" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A48" s="4">
+      <c r="I47" t="s">
+        <v>12</v>
+      </c>
+      <c r="J47" t="s">
+        <v>13</v>
+      </c>
+      <c r="K47" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="48" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A48">
         <v>6</v>
       </c>
-      <c r="B48" s="4" t="s">
+      <c r="B48" t="s">
         <v>22</v>
       </c>
-      <c r="C48" s="4">
+      <c r="C48">
         <v>5</v>
       </c>
-      <c r="D48" s="4">
+      <c r="D48">
         <v>20</v>
       </c>
-      <c r="E48" s="4">
-        <v>0</v>
-      </c>
-      <c r="F48" s="4">
-        <v>0</v>
-      </c>
-      <c r="G48" s="4">
-        <v>0</v>
-      </c>
-      <c r="H48" s="5">
+      <c r="E48">
+        <v>0</v>
+      </c>
+      <c r="F48">
+        <v>0</v>
+      </c>
+      <c r="G48">
+        <v>0</v>
+      </c>
+      <c r="H48">
         <v>78554</v>
       </c>
-      <c r="I48" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="J48" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="K48" s="4" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="49" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A49" s="4">
+      <c r="I48" t="s">
+        <v>12</v>
+      </c>
+      <c r="J48" t="s">
+        <v>13</v>
+      </c>
+      <c r="K48" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="49" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A49">
         <v>6</v>
       </c>
-      <c r="B49" s="4" t="s">
+      <c r="B49" t="s">
         <v>19</v>
       </c>
-      <c r="C49" s="4">
+      <c r="C49">
         <v>34</v>
       </c>
-      <c r="D49" s="4">
+      <c r="D49">
         <v>124</v>
       </c>
-      <c r="E49" s="4">
+      <c r="E49">
         <v>6</v>
       </c>
-      <c r="F49" s="4">
-        <v>0</v>
-      </c>
-      <c r="G49" s="4">
-        <v>0</v>
-      </c>
-      <c r="H49" s="5">
+      <c r="F49">
+        <v>0</v>
+      </c>
+      <c r="G49">
+        <v>0</v>
+      </c>
+      <c r="H49">
         <v>470362</v>
       </c>
-      <c r="I49" s="5">
+      <c r="I49">
         <v>8963</v>
       </c>
-      <c r="J49" s="5">
+      <c r="J49">
         <v>1984</v>
       </c>
-      <c r="K49" s="5">
+      <c r="K49">
         <v>26236</v>
       </c>
     </row>
-    <row r="50" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A50" s="4">
+    <row r="50" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A50">
         <v>7</v>
       </c>
-      <c r="B50" s="4" t="s">
+      <c r="B50" t="s">
         <v>28</v>
       </c>
-      <c r="C50" s="4">
-        <v>3</v>
-      </c>
-      <c r="D50" s="4">
-        <v>12</v>
-      </c>
-      <c r="E50" s="4">
-        <v>0</v>
-      </c>
-      <c r="F50" s="4">
-        <v>0</v>
-      </c>
-      <c r="G50" s="4">
-        <v>0</v>
-      </c>
-      <c r="H50" s="5">
+      <c r="C50">
+        <v>3</v>
+      </c>
+      <c r="D50">
+        <v>12</v>
+      </c>
+      <c r="E50">
+        <v>0</v>
+      </c>
+      <c r="F50">
+        <v>0</v>
+      </c>
+      <c r="G50">
+        <v>0</v>
+      </c>
+      <c r="H50">
         <v>53249</v>
       </c>
-      <c r="I50" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="J50" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="K50" s="4" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="51" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A51" s="4">
+      <c r="I50" t="s">
+        <v>12</v>
+      </c>
+      <c r="J50" t="s">
+        <v>13</v>
+      </c>
+      <c r="K50" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="51" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A51">
         <v>7</v>
       </c>
-      <c r="B51" s="4" t="s">
+      <c r="B51" t="s">
         <v>11</v>
       </c>
-      <c r="C51" s="4">
-        <v>0</v>
-      </c>
-      <c r="D51" s="4">
-        <v>0</v>
-      </c>
-      <c r="E51" s="4">
-        <v>0</v>
-      </c>
-      <c r="F51" s="4">
-        <v>0</v>
-      </c>
-      <c r="G51" s="4">
-        <v>0</v>
-      </c>
-      <c r="H51" s="4">
-        <v>0</v>
-      </c>
-      <c r="I51" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="J51" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="K51" s="4" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="52" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A52" s="4">
+      <c r="C51">
+        <v>0</v>
+      </c>
+      <c r="D51">
+        <v>0</v>
+      </c>
+      <c r="E51">
+        <v>0</v>
+      </c>
+      <c r="F51">
+        <v>0</v>
+      </c>
+      <c r="G51">
+        <v>0</v>
+      </c>
+      <c r="H51">
+        <v>0</v>
+      </c>
+      <c r="I51" t="s">
+        <v>13</v>
+      </c>
+      <c r="J51" t="s">
+        <v>13</v>
+      </c>
+      <c r="K51" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="52" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A52">
         <v>7</v>
       </c>
-      <c r="B52" s="4" t="s">
+      <c r="B52" t="s">
         <v>14</v>
       </c>
-      <c r="C52" s="4">
-        <v>0</v>
-      </c>
-      <c r="D52" s="4">
-        <v>0</v>
-      </c>
-      <c r="E52" s="4">
-        <v>0</v>
-      </c>
-      <c r="F52" s="4">
-        <v>0</v>
-      </c>
-      <c r="G52" s="4">
-        <v>0</v>
-      </c>
-      <c r="H52" s="4">
-        <v>0</v>
-      </c>
-      <c r="I52" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="J52" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="K52" s="4" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="53" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A53" s="4">
+      <c r="C52">
+        <v>0</v>
+      </c>
+      <c r="D52">
+        <v>0</v>
+      </c>
+      <c r="E52">
+        <v>0</v>
+      </c>
+      <c r="F52">
+        <v>0</v>
+      </c>
+      <c r="G52">
+        <v>0</v>
+      </c>
+      <c r="H52">
+        <v>0</v>
+      </c>
+      <c r="I52" t="s">
+        <v>13</v>
+      </c>
+      <c r="J52" t="s">
+        <v>13</v>
+      </c>
+      <c r="K52" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="53" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A53">
         <v>7</v>
       </c>
-      <c r="B53" s="4" t="s">
+      <c r="B53" t="s">
         <v>15</v>
       </c>
-      <c r="C53" s="4">
-        <v>3</v>
-      </c>
-      <c r="D53" s="4">
-        <v>12</v>
-      </c>
-      <c r="E53" s="4">
-        <v>0</v>
-      </c>
-      <c r="F53" s="4">
-        <v>0</v>
-      </c>
-      <c r="G53" s="4">
-        <v>0</v>
-      </c>
-      <c r="H53" s="5">
+      <c r="C53">
+        <v>3</v>
+      </c>
+      <c r="D53">
+        <v>12</v>
+      </c>
+      <c r="E53">
+        <v>0</v>
+      </c>
+      <c r="F53">
+        <v>0</v>
+      </c>
+      <c r="G53">
+        <v>0</v>
+      </c>
+      <c r="H53">
         <v>43072</v>
       </c>
-      <c r="I53" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="J53" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="K53" s="4" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="54" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A54" s="4">
+      <c r="I53" t="s">
+        <v>12</v>
+      </c>
+      <c r="J53" t="s">
+        <v>13</v>
+      </c>
+      <c r="K53" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="54" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A54">
         <v>7</v>
       </c>
-      <c r="B54" s="4" t="s">
+      <c r="B54" t="s">
         <v>16</v>
       </c>
-      <c r="C54" s="4">
-        <v>0</v>
-      </c>
-      <c r="D54" s="4">
-        <v>0</v>
-      </c>
-      <c r="E54" s="4">
-        <v>0</v>
-      </c>
-      <c r="F54" s="4">
-        <v>0</v>
-      </c>
-      <c r="G54" s="4">
-        <v>0</v>
-      </c>
-      <c r="H54" s="4">
-        <v>0</v>
-      </c>
-      <c r="I54" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="J54" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="K54" s="4" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="55" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A55" s="4">
+      <c r="C54">
+        <v>0</v>
+      </c>
+      <c r="D54">
+        <v>0</v>
+      </c>
+      <c r="E54">
+        <v>0</v>
+      </c>
+      <c r="F54">
+        <v>0</v>
+      </c>
+      <c r="G54">
+        <v>0</v>
+      </c>
+      <c r="H54">
+        <v>0</v>
+      </c>
+      <c r="I54" t="s">
+        <v>13</v>
+      </c>
+      <c r="J54" t="s">
+        <v>13</v>
+      </c>
+      <c r="K54" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="55" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A55">
         <v>7</v>
       </c>
-      <c r="B55" s="4" t="s">
+      <c r="B55" t="s">
         <v>17</v>
       </c>
-      <c r="C55" s="4">
-        <v>0</v>
-      </c>
-      <c r="D55" s="4">
-        <v>0</v>
-      </c>
-      <c r="E55" s="4">
-        <v>0</v>
-      </c>
-      <c r="F55" s="4">
-        <v>0</v>
-      </c>
-      <c r="G55" s="4">
-        <v>0</v>
-      </c>
-      <c r="H55" s="4">
-        <v>0</v>
-      </c>
-      <c r="I55" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="J55" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="K55" s="4" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="56" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A56" s="4">
+      <c r="C55">
+        <v>0</v>
+      </c>
+      <c r="D55">
+        <v>0</v>
+      </c>
+      <c r="E55">
+        <v>0</v>
+      </c>
+      <c r="F55">
+        <v>0</v>
+      </c>
+      <c r="G55">
+        <v>0</v>
+      </c>
+      <c r="H55">
+        <v>0</v>
+      </c>
+      <c r="I55" t="s">
+        <v>13</v>
+      </c>
+      <c r="J55" t="s">
+        <v>13</v>
+      </c>
+      <c r="K55" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="56" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A56">
         <v>7</v>
       </c>
-      <c r="B56" s="4" t="s">
+      <c r="B56" t="s">
         <v>18</v>
       </c>
-      <c r="C56" s="4">
-        <v>0</v>
-      </c>
-      <c r="D56" s="4">
-        <v>0</v>
-      </c>
-      <c r="E56" s="4">
-        <v>0</v>
-      </c>
-      <c r="F56" s="4">
-        <v>0</v>
-      </c>
-      <c r="G56" s="4">
-        <v>0</v>
-      </c>
-      <c r="H56" s="4">
-        <v>0</v>
-      </c>
-      <c r="I56" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="J56" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="K56" s="4" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="57" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A57" s="4">
+      <c r="C56">
+        <v>0</v>
+      </c>
+      <c r="D56">
+        <v>0</v>
+      </c>
+      <c r="E56">
+        <v>0</v>
+      </c>
+      <c r="F56">
+        <v>0</v>
+      </c>
+      <c r="G56">
+        <v>0</v>
+      </c>
+      <c r="H56">
+        <v>0</v>
+      </c>
+      <c r="I56" t="s">
+        <v>13</v>
+      </c>
+      <c r="J56" t="s">
+        <v>13</v>
+      </c>
+      <c r="K56" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="57" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A57">
         <v>7</v>
       </c>
-      <c r="B57" s="4" t="s">
+      <c r="B57" t="s">
         <v>22</v>
       </c>
-      <c r="C57" s="4">
-        <v>3</v>
-      </c>
-      <c r="D57" s="4">
-        <v>12</v>
-      </c>
-      <c r="E57" s="4">
-        <v>0</v>
-      </c>
-      <c r="F57" s="4">
-        <v>0</v>
-      </c>
-      <c r="G57" s="4">
-        <v>0</v>
-      </c>
-      <c r="H57" s="5">
+      <c r="C57">
+        <v>3</v>
+      </c>
+      <c r="D57">
+        <v>12</v>
+      </c>
+      <c r="E57">
+        <v>0</v>
+      </c>
+      <c r="F57">
+        <v>0</v>
+      </c>
+      <c r="G57">
+        <v>0</v>
+      </c>
+      <c r="H57">
         <v>41695</v>
       </c>
-      <c r="I57" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="J57" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="K57" s="4" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="58" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A58" s="4">
+      <c r="I57" t="s">
+        <v>12</v>
+      </c>
+      <c r="J57" t="s">
+        <v>13</v>
+      </c>
+      <c r="K57" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="58" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A58">
         <v>7</v>
       </c>
-      <c r="B58" s="4" t="s">
+      <c r="B58" t="s">
         <v>19</v>
       </c>
-      <c r="C58" s="4">
+      <c r="C58">
         <v>9</v>
       </c>
-      <c r="D58" s="4">
+      <c r="D58">
         <v>36</v>
       </c>
-      <c r="E58" s="4">
-        <v>0</v>
-      </c>
-      <c r="F58" s="4">
-        <v>0</v>
-      </c>
-      <c r="G58" s="4">
-        <v>0</v>
-      </c>
-      <c r="H58" s="5">
+      <c r="E58">
+        <v>0</v>
+      </c>
+      <c r="F58">
+        <v>0</v>
+      </c>
+      <c r="G58">
+        <v>0</v>
+      </c>
+      <c r="H58">
         <v>138016</v>
       </c>
-      <c r="I58" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="J58" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="K58" s="4" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="59" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A59" s="4">
+      <c r="I58" t="s">
+        <v>12</v>
+      </c>
+      <c r="J58" t="s">
+        <v>13</v>
+      </c>
+      <c r="K58" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="59" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A59">
         <v>8</v>
       </c>
-      <c r="B59" s="4" t="s">
+      <c r="B59" t="s">
         <v>28</v>
       </c>
-      <c r="C59" s="4">
-        <v>3</v>
-      </c>
-      <c r="D59" s="4">
-        <v>12</v>
-      </c>
-      <c r="E59" s="4">
-        <v>0</v>
-      </c>
-      <c r="F59" s="4">
-        <v>0</v>
-      </c>
-      <c r="G59" s="4">
-        <v>0</v>
-      </c>
-      <c r="H59" s="5">
+      <c r="C59">
+        <v>3</v>
+      </c>
+      <c r="D59">
+        <v>12</v>
+      </c>
+      <c r="E59">
+        <v>0</v>
+      </c>
+      <c r="F59">
+        <v>0</v>
+      </c>
+      <c r="G59">
+        <v>0</v>
+      </c>
+      <c r="H59">
         <v>59695</v>
       </c>
-      <c r="I59" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="J59" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="K59" s="4" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="60" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A60" s="4">
+      <c r="I59" t="s">
+        <v>12</v>
+      </c>
+      <c r="J59" t="s">
+        <v>13</v>
+      </c>
+      <c r="K59" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="60" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A60">
         <v>8</v>
       </c>
-      <c r="B60" s="4" t="s">
+      <c r="B60" t="s">
         <v>11</v>
       </c>
-      <c r="C60" s="4">
-        <v>3</v>
-      </c>
-      <c r="D60" s="4">
-        <v>12</v>
-      </c>
-      <c r="E60" s="4">
-        <v>0</v>
-      </c>
-      <c r="F60" s="4">
-        <v>0</v>
-      </c>
-      <c r="G60" s="4">
-        <v>0</v>
-      </c>
-      <c r="H60" s="5">
+      <c r="C60">
+        <v>3</v>
+      </c>
+      <c r="D60">
+        <v>12</v>
+      </c>
+      <c r="E60">
+        <v>0</v>
+      </c>
+      <c r="F60">
+        <v>0</v>
+      </c>
+      <c r="G60">
+        <v>0</v>
+      </c>
+      <c r="H60">
         <v>48484</v>
       </c>
-      <c r="I60" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="J60" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="K60" s="4" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="61" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A61" s="4">
+      <c r="I60" t="s">
+        <v>12</v>
+      </c>
+      <c r="J60" t="s">
+        <v>13</v>
+      </c>
+      <c r="K60" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="61" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A61">
         <v>8</v>
       </c>
-      <c r="B61" s="4" t="s">
+      <c r="B61" t="s">
         <v>14</v>
       </c>
-      <c r="C61" s="4">
-        <v>0</v>
-      </c>
-      <c r="D61" s="4">
-        <v>0</v>
-      </c>
-      <c r="E61" s="4">
-        <v>0</v>
-      </c>
-      <c r="F61" s="4">
-        <v>0</v>
-      </c>
-      <c r="G61" s="4">
-        <v>0</v>
-      </c>
-      <c r="H61" s="4">
-        <v>0</v>
-      </c>
-      <c r="I61" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="J61" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="K61" s="4" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="62" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A62" s="4">
+      <c r="C61">
+        <v>0</v>
+      </c>
+      <c r="D61">
+        <v>0</v>
+      </c>
+      <c r="E61">
+        <v>0</v>
+      </c>
+      <c r="F61">
+        <v>0</v>
+      </c>
+      <c r="G61">
+        <v>0</v>
+      </c>
+      <c r="H61">
+        <v>0</v>
+      </c>
+      <c r="I61" t="s">
+        <v>13</v>
+      </c>
+      <c r="J61" t="s">
+        <v>13</v>
+      </c>
+      <c r="K61" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="62" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A62">
         <v>8</v>
       </c>
-      <c r="B62" s="4" t="s">
+      <c r="B62" t="s">
         <v>15</v>
       </c>
-      <c r="C62" s="4">
-        <v>3</v>
-      </c>
-      <c r="D62" s="4">
-        <v>12</v>
-      </c>
-      <c r="E62" s="4">
-        <v>0</v>
-      </c>
-      <c r="F62" s="4">
-        <v>0</v>
-      </c>
-      <c r="G62" s="4">
-        <v>0</v>
-      </c>
-      <c r="H62" s="5">
+      <c r="C62">
+        <v>3</v>
+      </c>
+      <c r="D62">
+        <v>12</v>
+      </c>
+      <c r="E62">
+        <v>0</v>
+      </c>
+      <c r="F62">
+        <v>0</v>
+      </c>
+      <c r="G62">
+        <v>0</v>
+      </c>
+      <c r="H62">
         <v>52223</v>
       </c>
-      <c r="I62" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="J62" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="K62" s="4" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="63" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A63" s="4">
+      <c r="I62" t="s">
+        <v>12</v>
+      </c>
+      <c r="J62" t="s">
+        <v>13</v>
+      </c>
+      <c r="K62" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="63" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A63">
         <v>8</v>
       </c>
-      <c r="B63" s="4" t="s">
+      <c r="B63" t="s">
         <v>16</v>
       </c>
-      <c r="C63" s="4">
-        <v>0</v>
-      </c>
-      <c r="D63" s="4">
-        <v>0</v>
-      </c>
-      <c r="E63" s="4">
-        <v>0</v>
-      </c>
-      <c r="F63" s="4">
-        <v>0</v>
-      </c>
-      <c r="G63" s="4">
-        <v>0</v>
-      </c>
-      <c r="H63" s="4">
-        <v>0</v>
-      </c>
-      <c r="I63" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="J63" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="K63" s="4" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="64" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A64" s="4">
+      <c r="C63">
+        <v>0</v>
+      </c>
+      <c r="D63">
+        <v>0</v>
+      </c>
+      <c r="E63">
+        <v>0</v>
+      </c>
+      <c r="F63">
+        <v>0</v>
+      </c>
+      <c r="G63">
+        <v>0</v>
+      </c>
+      <c r="H63">
+        <v>0</v>
+      </c>
+      <c r="I63" t="s">
+        <v>13</v>
+      </c>
+      <c r="J63" t="s">
+        <v>13</v>
+      </c>
+      <c r="K63" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="64" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A64">
         <v>8</v>
       </c>
-      <c r="B64" s="4" t="s">
+      <c r="B64" t="s">
         <v>17</v>
       </c>
-      <c r="C64" s="4">
-        <v>3</v>
-      </c>
-      <c r="D64" s="4">
+      <c r="C64">
+        <v>3</v>
+      </c>
+      <c r="D64">
         <v>10</v>
       </c>
-      <c r="E64" s="4">
+      <c r="E64">
         <v>1</v>
       </c>
-      <c r="F64" s="4">
-        <v>0</v>
-      </c>
-      <c r="G64" s="4">
-        <v>0</v>
-      </c>
-      <c r="H64" s="5">
+      <c r="F64">
+        <v>0</v>
+      </c>
+      <c r="G64">
+        <v>0</v>
+      </c>
+      <c r="H64">
         <v>34478</v>
       </c>
-      <c r="I64" s="4">
+      <c r="I64">
         <v>258</v>
       </c>
-      <c r="J64" s="4">
+      <c r="J64">
         <v>16</v>
       </c>
-      <c r="K64" s="5">
+      <c r="K64">
         <v>1219</v>
       </c>
     </row>
-    <row r="65" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A65" s="4">
+    <row r="65" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A65">
         <v>8</v>
       </c>
-      <c r="B65" s="4" t="s">
+      <c r="B65" t="s">
         <v>18</v>
       </c>
-      <c r="C65" s="4">
+      <c r="C65">
         <v>6</v>
       </c>
-      <c r="D65" s="4">
+      <c r="D65">
         <v>24</v>
       </c>
-      <c r="E65" s="4">
-        <v>0</v>
-      </c>
-      <c r="F65" s="4">
-        <v>0</v>
-      </c>
-      <c r="G65" s="4">
-        <v>0</v>
-      </c>
-      <c r="H65" s="5">
+      <c r="E65">
+        <v>0</v>
+      </c>
+      <c r="F65">
+        <v>0</v>
+      </c>
+      <c r="G65">
+        <v>0</v>
+      </c>
+      <c r="H65">
         <v>81962</v>
       </c>
-      <c r="I65" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="J65" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="K65" s="4" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="66" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A66" s="4">
+      <c r="I65" t="s">
+        <v>12</v>
+      </c>
+      <c r="J65" t="s">
+        <v>13</v>
+      </c>
+      <c r="K65" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="66" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A66">
         <v>8</v>
       </c>
-      <c r="B66" s="4" t="s">
+      <c r="B66" t="s">
         <v>22</v>
       </c>
-      <c r="C66" s="4">
-        <v>3</v>
-      </c>
-      <c r="D66" s="4">
+      <c r="C66">
+        <v>3</v>
+      </c>
+      <c r="D66">
         <v>10</v>
       </c>
-      <c r="E66" s="4">
-        <v>0</v>
-      </c>
-      <c r="F66" s="4">
-        <v>0</v>
-      </c>
-      <c r="G66" s="4">
-        <v>0</v>
-      </c>
-      <c r="H66" s="5">
+      <c r="E66">
+        <v>0</v>
+      </c>
+      <c r="F66">
+        <v>0</v>
+      </c>
+      <c r="G66">
+        <v>0</v>
+      </c>
+      <c r="H66">
         <v>30268</v>
       </c>
-      <c r="I66" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="J66" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="K66" s="4" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="67" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A67" s="4">
+      <c r="I66" t="s">
+        <v>12</v>
+      </c>
+      <c r="J66" t="s">
+        <v>13</v>
+      </c>
+      <c r="K66" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="67" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A67">
         <v>8</v>
       </c>
-      <c r="B67" s="4" t="s">
+      <c r="B67" t="s">
         <v>19</v>
       </c>
-      <c r="C67" s="4">
+      <c r="C67">
         <v>21</v>
       </c>
-      <c r="D67" s="4">
+      <c r="D67">
         <v>80</v>
       </c>
-      <c r="E67" s="4">
+      <c r="E67">
         <v>1</v>
       </c>
-      <c r="F67" s="4">
-        <v>0</v>
-      </c>
-      <c r="G67" s="4">
-        <v>0</v>
-      </c>
-      <c r="H67" s="5">
+      <c r="F67">
+        <v>0</v>
+      </c>
+      <c r="G67">
+        <v>0</v>
+      </c>
+      <c r="H67">
         <v>307111</v>
       </c>
-      <c r="I67" s="4">
+      <c r="I67">
         <v>258</v>
       </c>
-      <c r="J67" s="4">
+      <c r="J67">
         <v>16</v>
       </c>
-      <c r="K67" s="5">
+      <c r="K67">
         <v>1219</v>
+      </c>
+    </row>
+    <row r="68" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A68">
+        <v>9</v>
+      </c>
+      <c r="B68" t="s">
+        <v>28</v>
+      </c>
+      <c r="C68">
+        <v>3</v>
+      </c>
+      <c r="D68">
+        <v>12</v>
+      </c>
+      <c r="E68">
+        <v>0</v>
+      </c>
+      <c r="F68">
+        <v>0</v>
+      </c>
+      <c r="G68">
+        <v>0</v>
+      </c>
+      <c r="H68" s="1">
+        <v>57132</v>
+      </c>
+      <c r="I68" t="s">
+        <v>12</v>
+      </c>
+      <c r="J68" t="s">
+        <v>13</v>
+      </c>
+      <c r="K68" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="69" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A69">
+        <v>9</v>
+      </c>
+      <c r="B69" t="s">
+        <v>11</v>
+      </c>
+      <c r="C69">
+        <v>6</v>
+      </c>
+      <c r="D69">
+        <v>24</v>
+      </c>
+      <c r="E69">
+        <v>0</v>
+      </c>
+      <c r="F69">
+        <v>0</v>
+      </c>
+      <c r="G69">
+        <v>0</v>
+      </c>
+      <c r="H69" s="1">
+        <v>106253</v>
+      </c>
+      <c r="I69" t="s">
+        <v>12</v>
+      </c>
+      <c r="J69" t="s">
+        <v>13</v>
+      </c>
+      <c r="K69" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="70" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A70">
+        <v>9</v>
+      </c>
+      <c r="B70" t="s">
+        <v>14</v>
+      </c>
+      <c r="C70">
+        <v>3</v>
+      </c>
+      <c r="D70">
+        <v>10</v>
+      </c>
+      <c r="E70">
+        <v>1</v>
+      </c>
+      <c r="F70">
+        <v>0</v>
+      </c>
+      <c r="G70">
+        <v>0</v>
+      </c>
+      <c r="H70" s="1">
+        <v>36441</v>
+      </c>
+      <c r="I70" s="1">
+        <v>2584</v>
+      </c>
+      <c r="J70">
+        <v>213</v>
+      </c>
+      <c r="K70" s="1">
+        <v>11257</v>
+      </c>
+    </row>
+    <row r="71" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A71">
+        <v>9</v>
+      </c>
+      <c r="B71" t="s">
+        <v>15</v>
+      </c>
+      <c r="C71">
+        <v>3</v>
+      </c>
+      <c r="D71">
+        <v>12</v>
+      </c>
+      <c r="E71">
+        <v>0</v>
+      </c>
+      <c r="F71">
+        <v>0</v>
+      </c>
+      <c r="G71">
+        <v>0</v>
+      </c>
+      <c r="H71" s="1">
+        <v>46153</v>
+      </c>
+      <c r="I71" t="s">
+        <v>12</v>
+      </c>
+      <c r="J71" t="s">
+        <v>13</v>
+      </c>
+      <c r="K71" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="72" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A72">
+        <v>9</v>
+      </c>
+      <c r="B72" t="s">
+        <v>16</v>
+      </c>
+      <c r="C72">
+        <v>3</v>
+      </c>
+      <c r="D72">
+        <v>12</v>
+      </c>
+      <c r="E72">
+        <v>0</v>
+      </c>
+      <c r="F72">
+        <v>0</v>
+      </c>
+      <c r="G72">
+        <v>0</v>
+      </c>
+      <c r="H72" s="1">
+        <v>48739</v>
+      </c>
+      <c r="I72" t="s">
+        <v>12</v>
+      </c>
+      <c r="J72" t="s">
+        <v>13</v>
+      </c>
+      <c r="K72" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="73" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A73">
+        <v>9</v>
+      </c>
+      <c r="B73" t="s">
+        <v>17</v>
+      </c>
+      <c r="C73">
+        <v>0</v>
+      </c>
+      <c r="D73">
+        <v>0</v>
+      </c>
+      <c r="E73">
+        <v>0</v>
+      </c>
+      <c r="F73">
+        <v>0</v>
+      </c>
+      <c r="G73">
+        <v>0</v>
+      </c>
+      <c r="H73">
+        <v>0</v>
+      </c>
+      <c r="I73" t="s">
+        <v>13</v>
+      </c>
+      <c r="J73" t="s">
+        <v>13</v>
+      </c>
+      <c r="K73" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="74" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A74">
+        <v>9</v>
+      </c>
+      <c r="B74" t="s">
+        <v>18</v>
+      </c>
+      <c r="C74">
+        <v>6</v>
+      </c>
+      <c r="D74">
+        <v>24</v>
+      </c>
+      <c r="E74">
+        <v>0</v>
+      </c>
+      <c r="F74">
+        <v>0</v>
+      </c>
+      <c r="G74">
+        <v>0</v>
+      </c>
+      <c r="H74" s="1">
+        <v>90039</v>
+      </c>
+      <c r="I74" t="s">
+        <v>12</v>
+      </c>
+      <c r="J74" t="s">
+        <v>13</v>
+      </c>
+      <c r="K74" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="75" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A75">
+        <v>9</v>
+      </c>
+      <c r="B75" t="s">
+        <v>22</v>
+      </c>
+      <c r="C75">
+        <v>3</v>
+      </c>
+      <c r="D75">
+        <v>12</v>
+      </c>
+      <c r="E75">
+        <v>0</v>
+      </c>
+      <c r="F75">
+        <v>0</v>
+      </c>
+      <c r="G75">
+        <v>0</v>
+      </c>
+      <c r="H75" s="1">
+        <v>44354</v>
+      </c>
+      <c r="I75" t="s">
+        <v>12</v>
+      </c>
+      <c r="J75" t="s">
+        <v>13</v>
+      </c>
+      <c r="K75" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="76" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A76">
+        <v>9</v>
+      </c>
+      <c r="B76" t="s">
+        <v>19</v>
+      </c>
+      <c r="C76">
+        <v>27</v>
+      </c>
+      <c r="D76">
+        <v>106</v>
+      </c>
+      <c r="E76">
+        <v>1</v>
+      </c>
+      <c r="F76">
+        <v>0</v>
+      </c>
+      <c r="G76">
+        <v>0</v>
+      </c>
+      <c r="H76" s="1">
+        <v>429112</v>
+      </c>
+      <c r="I76" s="1">
+        <v>2584</v>
+      </c>
+      <c r="J76">
+        <v>213</v>
+      </c>
+      <c r="K76" s="1">
+        <v>11257</v>
       </c>
     </row>
   </sheetData>
@@ -2895,83 +3189,91 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DC5A6928-3806-4082-94AB-A52936AB7317}">
-  <dimension ref="A1:B9"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:B10"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="27.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="5.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="27.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1" s="6" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="6" t="s">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A1" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="4" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A2" s="6">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A2">
         <v>1</v>
       </c>
-      <c r="B2" s="6" t="s">
+      <c r="B2" s="4" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A3" s="6">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A3">
         <v>2</v>
       </c>
-      <c r="B3" s="6" t="s">
+      <c r="B3" s="4" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A4" s="6">
-        <v>3</v>
-      </c>
-      <c r="B4" s="6" t="s">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4" s="4" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A5" s="6">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A5">
         <v>4</v>
       </c>
-      <c r="B5" s="6" t="s">
+      <c r="B5" s="4" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A6" s="6">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A6">
         <v>5</v>
       </c>
-      <c r="B6" s="6" t="s">
+      <c r="B6" s="4" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A7" s="7">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A7">
         <v>6</v>
       </c>
-      <c r="B7" s="7" t="s">
+      <c r="B7" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A8" s="7">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A8">
         <v>7</v>
       </c>
-      <c r="B8" s="8" t="s">
+      <c r="B8" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A9" s="7">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A9">
         <v>8</v>
       </c>
-      <c r="B9" s="8" t="s">
+      <c r="B9" t="s">
         <v>30</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A10">
+        <v>9</v>
+      </c>
+      <c r="B10" t="s">
+        <v>31</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Updates 2/9 for smelt assessment
</commit_message>
<xml_diff>
--- a/data_raw/smelt/abundance_estimates.xlsx
+++ b/data_raw/smelt/abundance_estimates.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://doimspp-my.sharepoint.com/personal/lmccormick_usbr_gov/Documents/Documents/Research/R/samt_smt_assessments/data_raw/smelt/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="94" documentId="8_{BF3B047A-36C0-4AD4-A0BA-7FD3D60567F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9C55109B-7597-4BD3-8F81-E592B50DADC1}"/>
+  <xr:revisionPtr revIDLastSave="98" documentId="8_{BF3B047A-36C0-4AD4-A0BA-7FD3D60567F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2D939A10-6EE7-4B20-B034-DE6D321C18BD}"/>
   <bookViews>
-    <workbookView xWindow="13680" yWindow="-14328" windowWidth="19584" windowHeight="11040" xr2:uid="{03E7A685-4EE0-4A4E-B4B4-B1F660F8462C}"/>
+    <workbookView xWindow="12084" yWindow="-15720" windowWidth="23040" windowHeight="12120" xr2:uid="{03E7A685-4EE0-4A4E-B4B4-B1F660F8462C}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="271" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="302" uniqueCount="33">
   <si>
     <t>Week</t>
   </si>
@@ -134,6 +134,9 @@
   <si>
     <t>January 26–30, 2026</t>
   </si>
+  <si>
+    <t>February 2–6, 2026</t>
+  </si>
 </sst>
 </file>
 
@@ -195,6 +198,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -514,7 +521,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{91E6CDBE-81F8-437E-8236-059C4BBF9395}">
-  <dimension ref="A1:K76"/>
+  <dimension ref="A1:K85"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="19.88671875" bestFit="1" customWidth="1"/>
@@ -3181,6 +3188,321 @@
         <v>11257</v>
       </c>
     </row>
+    <row r="77" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A77">
+        <v>10</v>
+      </c>
+      <c r="B77" t="s">
+        <v>28</v>
+      </c>
+      <c r="C77">
+        <v>0</v>
+      </c>
+      <c r="D77">
+        <v>0</v>
+      </c>
+      <c r="E77">
+        <v>0</v>
+      </c>
+      <c r="F77">
+        <v>0</v>
+      </c>
+      <c r="G77">
+        <v>0</v>
+      </c>
+      <c r="H77">
+        <v>0</v>
+      </c>
+      <c r="I77" t="s">
+        <v>13</v>
+      </c>
+      <c r="J77" t="s">
+        <v>13</v>
+      </c>
+      <c r="K77" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="78" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A78">
+        <v>10</v>
+      </c>
+      <c r="B78" t="s">
+        <v>11</v>
+      </c>
+      <c r="C78">
+        <v>3</v>
+      </c>
+      <c r="D78">
+        <v>12</v>
+      </c>
+      <c r="E78">
+        <v>0</v>
+      </c>
+      <c r="F78">
+        <v>0</v>
+      </c>
+      <c r="G78">
+        <v>0</v>
+      </c>
+      <c r="H78" s="1">
+        <v>59929</v>
+      </c>
+      <c r="I78" t="s">
+        <v>12</v>
+      </c>
+      <c r="J78" t="s">
+        <v>13</v>
+      </c>
+      <c r="K78" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="79" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A79">
+        <v>10</v>
+      </c>
+      <c r="B79" t="s">
+        <v>14</v>
+      </c>
+      <c r="C79">
+        <v>3</v>
+      </c>
+      <c r="D79">
+        <v>11</v>
+      </c>
+      <c r="E79">
+        <v>1</v>
+      </c>
+      <c r="F79">
+        <v>0</v>
+      </c>
+      <c r="G79">
+        <v>0</v>
+      </c>
+      <c r="H79" s="1">
+        <v>59197</v>
+      </c>
+      <c r="I79" s="1">
+        <v>1769</v>
+      </c>
+      <c r="J79">
+        <v>155</v>
+      </c>
+      <c r="K79" s="1">
+        <v>7562</v>
+      </c>
+    </row>
+    <row r="80" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A80">
+        <v>10</v>
+      </c>
+      <c r="B80" t="s">
+        <v>15</v>
+      </c>
+      <c r="C80">
+        <v>3</v>
+      </c>
+      <c r="D80">
+        <v>11</v>
+      </c>
+      <c r="E80">
+        <v>0</v>
+      </c>
+      <c r="F80">
+        <v>0</v>
+      </c>
+      <c r="G80">
+        <v>0</v>
+      </c>
+      <c r="H80" s="1">
+        <v>36521</v>
+      </c>
+      <c r="I80" t="s">
+        <v>12</v>
+      </c>
+      <c r="J80" t="s">
+        <v>13</v>
+      </c>
+      <c r="K80" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="81" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A81">
+        <v>10</v>
+      </c>
+      <c r="B81" t="s">
+        <v>16</v>
+      </c>
+      <c r="C81">
+        <v>3</v>
+      </c>
+      <c r="D81">
+        <v>12</v>
+      </c>
+      <c r="E81">
+        <v>0</v>
+      </c>
+      <c r="F81">
+        <v>0</v>
+      </c>
+      <c r="G81">
+        <v>0</v>
+      </c>
+      <c r="H81" s="1">
+        <v>42155</v>
+      </c>
+      <c r="I81" t="s">
+        <v>12</v>
+      </c>
+      <c r="J81" t="s">
+        <v>13</v>
+      </c>
+      <c r="K81" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="82" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A82">
+        <v>10</v>
+      </c>
+      <c r="B82" t="s">
+        <v>17</v>
+      </c>
+      <c r="C82">
+        <v>3</v>
+      </c>
+      <c r="D82">
+        <v>12</v>
+      </c>
+      <c r="E82">
+        <v>0</v>
+      </c>
+      <c r="F82">
+        <v>0</v>
+      </c>
+      <c r="G82">
+        <v>0</v>
+      </c>
+      <c r="H82" s="1">
+        <v>48916</v>
+      </c>
+      <c r="I82" t="s">
+        <v>12</v>
+      </c>
+      <c r="J82" t="s">
+        <v>13</v>
+      </c>
+      <c r="K82" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="83" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A83">
+        <v>10</v>
+      </c>
+      <c r="B83" t="s">
+        <v>18</v>
+      </c>
+      <c r="C83">
+        <v>3</v>
+      </c>
+      <c r="D83">
+        <v>12</v>
+      </c>
+      <c r="E83">
+        <v>0</v>
+      </c>
+      <c r="F83">
+        <v>0</v>
+      </c>
+      <c r="G83">
+        <v>0</v>
+      </c>
+      <c r="H83" s="1">
+        <v>46128</v>
+      </c>
+      <c r="I83" t="s">
+        <v>12</v>
+      </c>
+      <c r="J83" t="s">
+        <v>13</v>
+      </c>
+      <c r="K83" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="84" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A84">
+        <v>10</v>
+      </c>
+      <c r="B84" t="s">
+        <v>22</v>
+      </c>
+      <c r="C84">
+        <v>3</v>
+      </c>
+      <c r="D84">
+        <v>12</v>
+      </c>
+      <c r="E84">
+        <v>0</v>
+      </c>
+      <c r="F84">
+        <v>0</v>
+      </c>
+      <c r="G84">
+        <v>0</v>
+      </c>
+      <c r="H84" s="1">
+        <v>44498</v>
+      </c>
+      <c r="I84" t="s">
+        <v>12</v>
+      </c>
+      <c r="J84" t="s">
+        <v>13</v>
+      </c>
+      <c r="K84" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="85" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A85">
+        <v>10</v>
+      </c>
+      <c r="B85" t="s">
+        <v>19</v>
+      </c>
+      <c r="C85">
+        <v>21</v>
+      </c>
+      <c r="D85">
+        <v>82</v>
+      </c>
+      <c r="E85">
+        <v>1</v>
+      </c>
+      <c r="F85">
+        <v>0</v>
+      </c>
+      <c r="G85">
+        <v>0</v>
+      </c>
+      <c r="H85" s="1">
+        <v>337344</v>
+      </c>
+      <c r="I85" s="1">
+        <v>1769</v>
+      </c>
+      <c r="J85">
+        <v>155</v>
+      </c>
+      <c r="K85" s="1">
+        <v>7562</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
@@ -3189,7 +3511,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DC5A6928-3806-4082-94AB-A52936AB7317}">
-  <dimension ref="A1:B10"/>
+  <dimension ref="A1:B11"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="5.6640625" bestFit="1" customWidth="1"/>
@@ -3276,6 +3598,14 @@
         <v>31</v>
       </c>
     </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A11">
+        <v>10</v>
+      </c>
+      <c r="B11" t="s">
+        <v>32</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
Removed older files, added files 2/17
</commit_message>
<xml_diff>
--- a/data_raw/smelt/abundance_estimates.xlsx
+++ b/data_raw/smelt/abundance_estimates.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://doimspp-my.sharepoint.com/personal/lmccormick_usbr_gov/Documents/Documents/Research/R/samt_smt_assessments/data_raw/smelt/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="98" documentId="8_{BF3B047A-36C0-4AD4-A0BA-7FD3D60567F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2D939A10-6EE7-4B20-B034-DE6D321C18BD}"/>
+  <xr:revisionPtr revIDLastSave="102" documentId="8_{BF3B047A-36C0-4AD4-A0BA-7FD3D60567F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7B38FCB3-A24C-429A-9D26-854E75CA0175}"/>
   <bookViews>
-    <workbookView xWindow="12084" yWindow="-15720" windowWidth="23040" windowHeight="12120" xr2:uid="{03E7A685-4EE0-4A4E-B4B4-B1F660F8462C}"/>
+    <workbookView xWindow="12996" yWindow="-16032" windowWidth="17724" windowHeight="14964" xr2:uid="{03E7A685-4EE0-4A4E-B4B4-B1F660F8462C}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="302" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="333" uniqueCount="34">
   <si>
     <t>Week</t>
   </si>
@@ -136,6 +136,9 @@
   </si>
   <si>
     <t>February 2–6, 2026</t>
+  </si>
+  <si>
+    <t>February 9–13, 2026</t>
   </si>
 </sst>
 </file>
@@ -521,7 +524,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{91E6CDBE-81F8-437E-8236-059C4BBF9395}">
-  <dimension ref="A1:K85"/>
+  <dimension ref="A1:K94"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="19.88671875" bestFit="1" customWidth="1"/>
@@ -3503,6 +3506,321 @@
         <v>7562</v>
       </c>
     </row>
+    <row r="86" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A86">
+        <v>11</v>
+      </c>
+      <c r="B86" t="s">
+        <v>28</v>
+      </c>
+      <c r="C86">
+        <v>3</v>
+      </c>
+      <c r="D86">
+        <v>12</v>
+      </c>
+      <c r="E86">
+        <v>0</v>
+      </c>
+      <c r="F86">
+        <v>0</v>
+      </c>
+      <c r="G86">
+        <v>0</v>
+      </c>
+      <c r="H86" s="1">
+        <v>85729</v>
+      </c>
+      <c r="I86" t="s">
+        <v>12</v>
+      </c>
+      <c r="J86" t="s">
+        <v>13</v>
+      </c>
+      <c r="K86" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="87" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A87">
+        <v>11</v>
+      </c>
+      <c r="B87" t="s">
+        <v>11</v>
+      </c>
+      <c r="C87">
+        <v>6</v>
+      </c>
+      <c r="D87">
+        <v>22</v>
+      </c>
+      <c r="E87">
+        <v>0</v>
+      </c>
+      <c r="F87">
+        <v>0</v>
+      </c>
+      <c r="G87">
+        <v>0</v>
+      </c>
+      <c r="H87" s="1">
+        <v>116208</v>
+      </c>
+      <c r="I87" t="s">
+        <v>12</v>
+      </c>
+      <c r="J87" t="s">
+        <v>13</v>
+      </c>
+      <c r="K87" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="88" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A88">
+        <v>11</v>
+      </c>
+      <c r="B88" t="s">
+        <v>14</v>
+      </c>
+      <c r="C88">
+        <v>3</v>
+      </c>
+      <c r="D88">
+        <v>10</v>
+      </c>
+      <c r="E88">
+        <v>4</v>
+      </c>
+      <c r="F88">
+        <v>0</v>
+      </c>
+      <c r="G88">
+        <v>0</v>
+      </c>
+      <c r="H88" s="1">
+        <v>49313</v>
+      </c>
+      <c r="I88" s="1">
+        <v>4983</v>
+      </c>
+      <c r="J88">
+        <v>589</v>
+      </c>
+      <c r="K88" s="1">
+        <v>19146</v>
+      </c>
+    </row>
+    <row r="89" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A89">
+        <v>11</v>
+      </c>
+      <c r="B89" t="s">
+        <v>15</v>
+      </c>
+      <c r="C89">
+        <v>6</v>
+      </c>
+      <c r="D89">
+        <v>24</v>
+      </c>
+      <c r="E89">
+        <v>0</v>
+      </c>
+      <c r="F89">
+        <v>0</v>
+      </c>
+      <c r="G89">
+        <v>0</v>
+      </c>
+      <c r="H89" s="1">
+        <v>96054</v>
+      </c>
+      <c r="I89" t="s">
+        <v>12</v>
+      </c>
+      <c r="J89" t="s">
+        <v>13</v>
+      </c>
+      <c r="K89" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="90" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A90">
+        <v>11</v>
+      </c>
+      <c r="B90" t="s">
+        <v>16</v>
+      </c>
+      <c r="C90">
+        <v>3</v>
+      </c>
+      <c r="D90">
+        <v>10</v>
+      </c>
+      <c r="E90">
+        <v>0</v>
+      </c>
+      <c r="F90">
+        <v>0</v>
+      </c>
+      <c r="G90">
+        <v>0</v>
+      </c>
+      <c r="H90" s="1">
+        <v>36485</v>
+      </c>
+      <c r="I90" t="s">
+        <v>12</v>
+      </c>
+      <c r="J90" t="s">
+        <v>13</v>
+      </c>
+      <c r="K90" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="91" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A91">
+        <v>11</v>
+      </c>
+      <c r="B91" t="s">
+        <v>17</v>
+      </c>
+      <c r="C91">
+        <v>3</v>
+      </c>
+      <c r="D91">
+        <v>12</v>
+      </c>
+      <c r="E91">
+        <v>0</v>
+      </c>
+      <c r="F91">
+        <v>0</v>
+      </c>
+      <c r="G91">
+        <v>0</v>
+      </c>
+      <c r="H91" s="1">
+        <v>44795</v>
+      </c>
+      <c r="I91" t="s">
+        <v>12</v>
+      </c>
+      <c r="J91" t="s">
+        <v>13</v>
+      </c>
+      <c r="K91" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="92" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A92">
+        <v>11</v>
+      </c>
+      <c r="B92" t="s">
+        <v>18</v>
+      </c>
+      <c r="C92">
+        <v>6</v>
+      </c>
+      <c r="D92">
+        <v>24</v>
+      </c>
+      <c r="E92">
+        <v>0</v>
+      </c>
+      <c r="F92">
+        <v>0</v>
+      </c>
+      <c r="G92">
+        <v>0</v>
+      </c>
+      <c r="H92" s="1">
+        <v>97896</v>
+      </c>
+      <c r="I92" t="s">
+        <v>12</v>
+      </c>
+      <c r="J92" t="s">
+        <v>13</v>
+      </c>
+      <c r="K92" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="93" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A93">
+        <v>11</v>
+      </c>
+      <c r="B93" t="s">
+        <v>22</v>
+      </c>
+      <c r="C93">
+        <v>5</v>
+      </c>
+      <c r="D93">
+        <v>20</v>
+      </c>
+      <c r="E93">
+        <v>0</v>
+      </c>
+      <c r="F93">
+        <v>0</v>
+      </c>
+      <c r="G93">
+        <v>0</v>
+      </c>
+      <c r="H93" s="1">
+        <v>77757</v>
+      </c>
+      <c r="I93" t="s">
+        <v>12</v>
+      </c>
+      <c r="J93" t="s">
+        <v>13</v>
+      </c>
+      <c r="K93" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="94" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A94">
+        <v>11</v>
+      </c>
+      <c r="B94" t="s">
+        <v>19</v>
+      </c>
+      <c r="C94">
+        <v>35</v>
+      </c>
+      <c r="D94">
+        <v>134</v>
+      </c>
+      <c r="E94">
+        <v>4</v>
+      </c>
+      <c r="F94">
+        <v>0</v>
+      </c>
+      <c r="G94">
+        <v>0</v>
+      </c>
+      <c r="H94" s="1">
+        <v>604238</v>
+      </c>
+      <c r="I94" s="1">
+        <v>4983</v>
+      </c>
+      <c r="J94">
+        <v>589</v>
+      </c>
+      <c r="K94" s="1">
+        <v>19146</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
@@ -3511,7 +3829,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DC5A6928-3806-4082-94AB-A52936AB7317}">
-  <dimension ref="A1:B11"/>
+  <dimension ref="A1:B12"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="5.6640625" bestFit="1" customWidth="1"/>
@@ -3606,6 +3924,14 @@
         <v>32</v>
       </c>
     </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A12">
+        <v>11</v>
+      </c>
+      <c r="B12" t="s">
+        <v>33</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
Assessment edits 3/9/26. Manual salvage update.
</commit_message>
<xml_diff>
--- a/data_raw/smelt/abundance_estimates.xlsx
+++ b/data_raw/smelt/abundance_estimates.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://doimspp-my.sharepoint.com/personal/lmccormick_usbr_gov/Documents/Documents/Research/R/samt_smt_assessments/data_raw/smelt/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="110" documentId="8_{BF3B047A-36C0-4AD4-A0BA-7FD3D60567F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{40BE91BA-A548-4BC9-A2A4-ED9A996C5F9C}"/>
+  <xr:revisionPtr revIDLastSave="114" documentId="8_{BF3B047A-36C0-4AD4-A0BA-7FD3D60567F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{51CAAB37-4F6B-4395-8DB2-7F8E84E5A8D0}"/>
   <bookViews>
-    <workbookView xWindow="-18684" yWindow="-16188" windowWidth="23040" windowHeight="12120" xr2:uid="{03E7A685-4EE0-4A4E-B4B4-B1F660F8462C}"/>
+    <workbookView xWindow="11760" yWindow="-16200" windowWidth="25944" windowHeight="15144" xr2:uid="{03E7A685-4EE0-4A4E-B4B4-B1F660F8462C}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="401" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="432" uniqueCount="37">
   <si>
     <t>Week</t>
   </si>
@@ -145,6 +145,9 @@
   </si>
   <si>
     <t>February 23–27, 2026</t>
+  </si>
+  <si>
+    <t>March 2–6, 2026</t>
   </si>
 </sst>
 </file>
@@ -530,7 +533,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{91E6CDBE-81F8-437E-8236-059C4BBF9395}">
-  <dimension ref="A1:K112"/>
+  <dimension ref="A1:K121"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="19.88671875" bestFit="1" customWidth="1"/>
@@ -4457,6 +4460,321 @@
         <v>35401</v>
       </c>
     </row>
+    <row r="113" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A113">
+        <v>14</v>
+      </c>
+      <c r="B113" t="s">
+        <v>28</v>
+      </c>
+      <c r="C113">
+        <v>3</v>
+      </c>
+      <c r="D113">
+        <v>10</v>
+      </c>
+      <c r="E113">
+        <v>0</v>
+      </c>
+      <c r="F113">
+        <v>0</v>
+      </c>
+      <c r="G113">
+        <v>0</v>
+      </c>
+      <c r="H113" s="1">
+        <v>49465</v>
+      </c>
+      <c r="I113" t="s">
+        <v>12</v>
+      </c>
+      <c r="J113" t="s">
+        <v>13</v>
+      </c>
+      <c r="K113" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="114" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A114">
+        <v>14</v>
+      </c>
+      <c r="B114" t="s">
+        <v>11</v>
+      </c>
+      <c r="C114">
+        <v>5</v>
+      </c>
+      <c r="D114">
+        <v>20</v>
+      </c>
+      <c r="E114">
+        <v>0</v>
+      </c>
+      <c r="F114">
+        <v>0</v>
+      </c>
+      <c r="G114">
+        <v>0</v>
+      </c>
+      <c r="H114" s="1">
+        <v>104858</v>
+      </c>
+      <c r="I114" t="s">
+        <v>12</v>
+      </c>
+      <c r="J114" t="s">
+        <v>13</v>
+      </c>
+      <c r="K114" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="115" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A115">
+        <v>14</v>
+      </c>
+      <c r="B115" t="s">
+        <v>14</v>
+      </c>
+      <c r="C115">
+        <v>3</v>
+      </c>
+      <c r="D115">
+        <v>12</v>
+      </c>
+      <c r="E115">
+        <v>1</v>
+      </c>
+      <c r="F115">
+        <v>0</v>
+      </c>
+      <c r="G115">
+        <v>0</v>
+      </c>
+      <c r="H115" s="1">
+        <v>58256</v>
+      </c>
+      <c r="I115" s="1">
+        <v>1487</v>
+      </c>
+      <c r="J115">
+        <v>118</v>
+      </c>
+      <c r="K115" s="1">
+        <v>6560</v>
+      </c>
+    </row>
+    <row r="116" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A116">
+        <v>14</v>
+      </c>
+      <c r="B116" t="s">
+        <v>15</v>
+      </c>
+      <c r="C116">
+        <v>5</v>
+      </c>
+      <c r="D116">
+        <v>20</v>
+      </c>
+      <c r="E116">
+        <v>0</v>
+      </c>
+      <c r="F116">
+        <v>0</v>
+      </c>
+      <c r="G116">
+        <v>0</v>
+      </c>
+      <c r="H116" s="1">
+        <v>80933</v>
+      </c>
+      <c r="I116" t="s">
+        <v>12</v>
+      </c>
+      <c r="J116" t="s">
+        <v>13</v>
+      </c>
+      <c r="K116" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="117" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A117">
+        <v>14</v>
+      </c>
+      <c r="B117" t="s">
+        <v>16</v>
+      </c>
+      <c r="C117">
+        <v>3</v>
+      </c>
+      <c r="D117">
+        <v>11</v>
+      </c>
+      <c r="E117">
+        <v>0</v>
+      </c>
+      <c r="F117">
+        <v>0</v>
+      </c>
+      <c r="G117">
+        <v>0</v>
+      </c>
+      <c r="H117" s="1">
+        <v>43706</v>
+      </c>
+      <c r="I117" t="s">
+        <v>12</v>
+      </c>
+      <c r="J117" t="s">
+        <v>13</v>
+      </c>
+      <c r="K117" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="118" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A118">
+        <v>14</v>
+      </c>
+      <c r="B118" t="s">
+        <v>17</v>
+      </c>
+      <c r="C118">
+        <v>3</v>
+      </c>
+      <c r="D118">
+        <v>12</v>
+      </c>
+      <c r="E118">
+        <v>0</v>
+      </c>
+      <c r="F118">
+        <v>0</v>
+      </c>
+      <c r="G118">
+        <v>0</v>
+      </c>
+      <c r="H118" s="1">
+        <v>44939</v>
+      </c>
+      <c r="I118" t="s">
+        <v>12</v>
+      </c>
+      <c r="J118" t="s">
+        <v>13</v>
+      </c>
+      <c r="K118" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="119" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A119">
+        <v>14</v>
+      </c>
+      <c r="B119" t="s">
+        <v>18</v>
+      </c>
+      <c r="C119">
+        <v>6</v>
+      </c>
+      <c r="D119">
+        <v>24</v>
+      </c>
+      <c r="E119">
+        <v>0</v>
+      </c>
+      <c r="F119">
+        <v>0</v>
+      </c>
+      <c r="G119">
+        <v>0</v>
+      </c>
+      <c r="H119" s="1">
+        <v>92099</v>
+      </c>
+      <c r="I119" t="s">
+        <v>12</v>
+      </c>
+      <c r="J119" t="s">
+        <v>13</v>
+      </c>
+      <c r="K119" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="120" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A120">
+        <v>14</v>
+      </c>
+      <c r="B120" t="s">
+        <v>22</v>
+      </c>
+      <c r="C120">
+        <v>5</v>
+      </c>
+      <c r="D120">
+        <v>20</v>
+      </c>
+      <c r="E120">
+        <v>0</v>
+      </c>
+      <c r="F120">
+        <v>0</v>
+      </c>
+      <c r="G120">
+        <v>0</v>
+      </c>
+      <c r="H120" s="1">
+        <v>71336</v>
+      </c>
+      <c r="I120" t="s">
+        <v>12</v>
+      </c>
+      <c r="J120" t="s">
+        <v>13</v>
+      </c>
+      <c r="K120" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="121" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A121">
+        <v>14</v>
+      </c>
+      <c r="B121" t="s">
+        <v>19</v>
+      </c>
+      <c r="C121">
+        <v>33</v>
+      </c>
+      <c r="D121">
+        <v>129</v>
+      </c>
+      <c r="E121">
+        <v>1</v>
+      </c>
+      <c r="F121">
+        <v>0</v>
+      </c>
+      <c r="G121">
+        <v>0</v>
+      </c>
+      <c r="H121" s="1">
+        <v>545592</v>
+      </c>
+      <c r="I121" s="1">
+        <v>1487</v>
+      </c>
+      <c r="J121">
+        <v>118</v>
+      </c>
+      <c r="K121" s="1">
+        <v>6560</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
@@ -4465,7 +4783,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DC5A6928-3806-4082-94AB-A52936AB7317}">
-  <dimension ref="A1:B14"/>
+  <dimension ref="A1:B15"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="5.6640625" bestFit="1" customWidth="1"/>
@@ -4584,6 +4902,14 @@
         <v>35</v>
       </c>
     </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A15">
+        <v>14</v>
+      </c>
+      <c r="B15" t="s">
+        <v>36</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
update EDSM abundance estimates
</commit_message>
<xml_diff>
--- a/data_raw/smelt/abundance_estimates.xlsx
+++ b/data_raw/smelt/abundance_estimates.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://doimspp-my.sharepoint.com/personal/lmccormick_usbr_gov/Documents/Documents/Research/R/samt_smt_assessments/data_raw/smelt/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://doimspp-my.sharepoint.com/personal/geasterbrook_usbr_gov/Documents/My Projects/SMT/Assessment/samt_smt_assessments/data_raw/smelt/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="122" documentId="8_{BF3B047A-36C0-4AD4-A0BA-7FD3D60567F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FBA22CD4-978D-4559-BAA0-F65628D81232}"/>
+  <xr:revisionPtr revIDLastSave="129" documentId="8_{BF3B047A-36C0-4AD4-A0BA-7FD3D60567F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BE73FAD4-FB2D-4001-8C01-A04F289A7F22}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="21672" windowHeight="11580" activeTab="1" xr2:uid="{03E7A685-4EE0-4A4E-B4B4-B1F660F8462C}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{03E7A685-4EE0-4A4E-B4B4-B1F660F8462C}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="463" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="494" uniqueCount="39">
   <si>
     <t>Week</t>
   </si>
@@ -152,12 +152,15 @@
   <si>
     <t>March 9–13, 2026</t>
   </si>
+  <si>
+    <t>March 16–20, 2026</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -165,13 +168,25 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -186,7 +201,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -197,6 +212,18 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -532,14 +559,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{91E6CDBE-81F8-437E-8236-059C4BBF9395}">
-  <dimension ref="A1:K130"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:K139"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="19.88671875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="16.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="19.85546875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="16.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -574,7 +601,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
@@ -609,7 +636,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>1</v>
       </c>
@@ -644,7 +671,7 @@
         <v>10740</v>
       </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>1</v>
       </c>
@@ -679,7 +706,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>1</v>
       </c>
@@ -714,7 +741,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>1</v>
       </c>
@@ -749,7 +776,7 @@
         <v>3065</v>
       </c>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>1</v>
       </c>
@@ -784,7 +811,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>1</v>
       </c>
@@ -819,7 +846,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>1</v>
       </c>
@@ -854,7 +881,7 @@
         <v>12103</v>
       </c>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>2</v>
       </c>
@@ -889,7 +916,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>2</v>
       </c>
@@ -924,7 +951,7 @@
         <v>29101</v>
       </c>
     </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>2</v>
       </c>
@@ -959,7 +986,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>2</v>
       </c>
@@ -994,7 +1021,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>2</v>
       </c>
@@ -1029,7 +1056,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>2</v>
       </c>
@@ -1064,7 +1091,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>2</v>
       </c>
@@ -1099,7 +1126,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>2</v>
       </c>
@@ -1134,7 +1161,7 @@
         <v>29101</v>
       </c>
     </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>3</v>
       </c>
@@ -1169,7 +1196,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>3</v>
       </c>
@@ -1204,7 +1231,7 @@
         <v>8836</v>
       </c>
     </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>3</v>
       </c>
@@ -1239,7 +1266,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>3</v>
       </c>
@@ -1274,7 +1301,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>3</v>
       </c>
@@ -1309,7 +1336,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A23">
         <v>3</v>
       </c>
@@ -1344,7 +1371,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>3</v>
       </c>
@@ -1379,7 +1406,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A25">
         <v>3</v>
       </c>
@@ -1414,7 +1441,7 @@
         <v>8836</v>
       </c>
     </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A26">
         <v>4</v>
       </c>
@@ -1449,7 +1476,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A27">
         <v>4</v>
       </c>
@@ -1484,7 +1511,7 @@
         <v>11902</v>
       </c>
     </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A28">
         <v>4</v>
       </c>
@@ -1519,7 +1546,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="29" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A29">
         <v>4</v>
       </c>
@@ -1554,7 +1581,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="30" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A30">
         <v>4</v>
       </c>
@@ -1589,7 +1616,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="31" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A31">
         <v>4</v>
       </c>
@@ -1624,7 +1651,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="32" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A32">
         <v>4</v>
       </c>
@@ -1659,7 +1686,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="33" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A33">
         <v>4</v>
       </c>
@@ -1694,7 +1721,7 @@
         <v>11902</v>
       </c>
     </row>
-    <row r="34" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A34">
         <v>5</v>
       </c>
@@ -1729,7 +1756,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="35" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A35">
         <v>5</v>
       </c>
@@ -1764,7 +1791,7 @@
         <v>20185</v>
       </c>
     </row>
-    <row r="36" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A36">
         <v>5</v>
       </c>
@@ -1799,7 +1826,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="37" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A37">
         <v>5</v>
       </c>
@@ -1834,7 +1861,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="38" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A38">
         <v>5</v>
       </c>
@@ -1869,7 +1896,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="39" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A39">
         <v>5</v>
       </c>
@@ -1904,7 +1931,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="40" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A40">
         <v>5</v>
       </c>
@@ -1939,7 +1966,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="41" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A41" s="2">
         <v>5</v>
       </c>
@@ -1974,7 +2001,7 @@
         <v>20185</v>
       </c>
     </row>
-    <row r="42" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A42">
         <v>6</v>
       </c>
@@ -2009,7 +2036,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="43" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A43">
         <v>6</v>
       </c>
@@ -2044,7 +2071,7 @@
         <v>26236</v>
       </c>
     </row>
-    <row r="44" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A44">
         <v>6</v>
       </c>
@@ -2079,7 +2106,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="45" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A45">
         <v>6</v>
       </c>
@@ -2114,7 +2141,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="46" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A46">
         <v>6</v>
       </c>
@@ -2149,7 +2176,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="47" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A47">
         <v>6</v>
       </c>
@@ -2184,7 +2211,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="48" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A48">
         <v>6</v>
       </c>
@@ -2219,7 +2246,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="49" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A49">
         <v>6</v>
       </c>
@@ -2254,7 +2281,7 @@
         <v>26236</v>
       </c>
     </row>
-    <row r="50" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A50">
         <v>7</v>
       </c>
@@ -2289,7 +2316,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="51" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A51">
         <v>7</v>
       </c>
@@ -2324,7 +2351,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="52" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A52">
         <v>7</v>
       </c>
@@ -2359,7 +2386,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="53" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A53">
         <v>7</v>
       </c>
@@ -2394,7 +2421,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="54" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A54">
         <v>7</v>
       </c>
@@ -2429,7 +2456,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="55" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A55">
         <v>7</v>
       </c>
@@ -2464,7 +2491,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="56" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A56">
         <v>7</v>
       </c>
@@ -2499,7 +2526,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="57" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A57">
         <v>7</v>
       </c>
@@ -2534,7 +2561,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="58" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A58">
         <v>7</v>
       </c>
@@ -2569,7 +2596,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="59" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A59">
         <v>8</v>
       </c>
@@ -2604,7 +2631,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="60" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A60">
         <v>8</v>
       </c>
@@ -2639,7 +2666,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="61" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A61">
         <v>8</v>
       </c>
@@ -2674,7 +2701,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="62" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A62">
         <v>8</v>
       </c>
@@ -2709,7 +2736,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="63" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A63">
         <v>8</v>
       </c>
@@ -2744,7 +2771,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="64" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A64">
         <v>8</v>
       </c>
@@ -2779,7 +2806,7 @@
         <v>1219</v>
       </c>
     </row>
-    <row r="65" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A65">
         <v>8</v>
       </c>
@@ -2814,7 +2841,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="66" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A66">
         <v>8</v>
       </c>
@@ -2849,7 +2876,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="67" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A67">
         <v>8</v>
       </c>
@@ -2884,7 +2911,7 @@
         <v>1219</v>
       </c>
     </row>
-    <row r="68" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A68">
         <v>9</v>
       </c>
@@ -2919,7 +2946,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="69" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A69">
         <v>9</v>
       </c>
@@ -2954,7 +2981,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="70" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A70">
         <v>9</v>
       </c>
@@ -2989,7 +3016,7 @@
         <v>11257</v>
       </c>
     </row>
-    <row r="71" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A71">
         <v>9</v>
       </c>
@@ -3024,7 +3051,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="72" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A72">
         <v>9</v>
       </c>
@@ -3059,7 +3086,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="73" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A73">
         <v>9</v>
       </c>
@@ -3094,7 +3121,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="74" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A74">
         <v>9</v>
       </c>
@@ -3129,7 +3156,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="75" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A75">
         <v>9</v>
       </c>
@@ -3164,7 +3191,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="76" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A76">
         <v>9</v>
       </c>
@@ -3199,7 +3226,7 @@
         <v>11257</v>
       </c>
     </row>
-    <row r="77" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A77">
         <v>10</v>
       </c>
@@ -3234,7 +3261,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="78" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A78">
         <v>10</v>
       </c>
@@ -3269,7 +3296,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="79" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A79">
         <v>10</v>
       </c>
@@ -3304,7 +3331,7 @@
         <v>7562</v>
       </c>
     </row>
-    <row r="80" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A80">
         <v>10</v>
       </c>
@@ -3339,7 +3366,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="81" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A81">
         <v>10</v>
       </c>
@@ -3374,7 +3401,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="82" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A82">
         <v>10</v>
       </c>
@@ -3409,7 +3436,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="83" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A83">
         <v>10</v>
       </c>
@@ -3444,7 +3471,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="84" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A84">
         <v>10</v>
       </c>
@@ -3479,7 +3506,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="85" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A85">
         <v>10</v>
       </c>
@@ -3514,7 +3541,7 @@
         <v>7562</v>
       </c>
     </row>
-    <row r="86" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A86">
         <v>11</v>
       </c>
@@ -3549,7 +3576,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="87" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A87">
         <v>11</v>
       </c>
@@ -3584,7 +3611,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="88" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A88">
         <v>11</v>
       </c>
@@ -3619,7 +3646,7 @@
         <v>19146</v>
       </c>
     </row>
-    <row r="89" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A89">
         <v>11</v>
       </c>
@@ -3654,7 +3681,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="90" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A90">
         <v>11</v>
       </c>
@@ -3689,7 +3716,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="91" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A91">
         <v>11</v>
       </c>
@@ -3724,7 +3751,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="92" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A92">
         <v>11</v>
       </c>
@@ -3759,7 +3786,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="93" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A93">
         <v>11</v>
       </c>
@@ -3794,7 +3821,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="94" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A94">
         <v>11</v>
       </c>
@@ -3829,7 +3856,7 @@
         <v>19146</v>
       </c>
     </row>
-    <row r="95" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A95">
         <v>12</v>
       </c>
@@ -3864,7 +3891,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="96" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A96">
         <v>12</v>
       </c>
@@ -3899,7 +3926,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="97" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A97">
         <v>12</v>
       </c>
@@ -3934,7 +3961,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="98" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A98">
         <v>12</v>
       </c>
@@ -3969,7 +3996,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="99" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A99">
         <v>12</v>
       </c>
@@ -4004,7 +4031,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="100" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A100">
         <v>12</v>
       </c>
@@ -4039,7 +4066,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="101" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A101">
         <v>12</v>
       </c>
@@ -4074,7 +4101,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="102" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A102">
         <v>12</v>
       </c>
@@ -4109,7 +4136,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="103" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A103">
         <v>12</v>
       </c>
@@ -4144,7 +4171,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="104" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A104">
         <v>13</v>
       </c>
@@ -4179,7 +4206,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="105" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A105">
         <v>13</v>
       </c>
@@ -4214,7 +4241,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="106" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="106" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A106">
         <v>13</v>
       </c>
@@ -4249,7 +4276,7 @@
         <v>35401</v>
       </c>
     </row>
-    <row r="107" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="107" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A107">
         <v>13</v>
       </c>
@@ -4284,7 +4311,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="108" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A108">
         <v>13</v>
       </c>
@@ -4319,7 +4346,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="109" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A109">
         <v>13</v>
       </c>
@@ -4354,7 +4381,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="110" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="110" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A110">
         <v>13</v>
       </c>
@@ -4389,7 +4416,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="111" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="111" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A111">
         <v>13</v>
       </c>
@@ -4424,7 +4451,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="112" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A112">
         <v>13</v>
       </c>
@@ -4459,7 +4486,7 @@
         <v>35401</v>
       </c>
     </row>
-    <row r="113" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="113" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A113">
         <v>14</v>
       </c>
@@ -4494,7 +4521,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="114" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="114" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A114">
         <v>14</v>
       </c>
@@ -4529,7 +4556,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="115" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="115" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A115">
         <v>14</v>
       </c>
@@ -4564,7 +4591,7 @@
         <v>6560</v>
       </c>
     </row>
-    <row r="116" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="116" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A116">
         <v>14</v>
       </c>
@@ -4599,7 +4626,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="117" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="117" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A117">
         <v>14</v>
       </c>
@@ -4634,7 +4661,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="118" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="118" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A118">
         <v>14</v>
       </c>
@@ -4669,7 +4696,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="119" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="119" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A119">
         <v>14</v>
       </c>
@@ -4704,7 +4731,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="120" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="120" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A120">
         <v>14</v>
       </c>
@@ -4739,7 +4766,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="121" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="121" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A121">
         <v>14</v>
       </c>
@@ -4774,7 +4801,7 @@
         <v>6560</v>
       </c>
     </row>
-    <row r="122" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="122" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A122">
         <v>15</v>
       </c>
@@ -4809,7 +4836,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="123" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="123" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A123">
         <v>15</v>
       </c>
@@ -4844,7 +4871,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="124" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="124" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A124">
         <v>15</v>
       </c>
@@ -4879,7 +4906,7 @@
         <v>8647</v>
       </c>
     </row>
-    <row r="125" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="125" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A125">
         <v>15</v>
       </c>
@@ -4914,7 +4941,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="126" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="126" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A126">
         <v>15</v>
       </c>
@@ -4949,7 +4976,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="127" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="127" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A127">
         <v>15</v>
       </c>
@@ -4984,7 +5011,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="128" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="128" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A128">
         <v>15</v>
       </c>
@@ -5019,7 +5046,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="129" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="129" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A129">
         <v>15</v>
       </c>
@@ -5054,7 +5081,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="130" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="130" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A130">
         <v>15</v>
       </c>
@@ -5087,6 +5114,321 @@
       </c>
       <c r="K130">
         <v>8647</v>
+      </c>
+    </row>
+    <row r="131" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A131" s="6">
+        <v>16</v>
+      </c>
+      <c r="B131" s="8" t="s">
+        <v>28</v>
+      </c>
+      <c r="C131" s="6">
+        <v>3</v>
+      </c>
+      <c r="D131" s="6">
+        <v>12</v>
+      </c>
+      <c r="E131" s="6">
+        <v>0</v>
+      </c>
+      <c r="F131" s="6">
+        <v>0</v>
+      </c>
+      <c r="G131" s="6">
+        <v>0</v>
+      </c>
+      <c r="H131" s="7">
+        <v>51975</v>
+      </c>
+      <c r="I131" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="J131" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="K131" s="6" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="132" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A132" s="6">
+        <v>16</v>
+      </c>
+      <c r="B132" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="C132" s="6">
+        <v>6</v>
+      </c>
+      <c r="D132" s="6">
+        <v>24</v>
+      </c>
+      <c r="E132" s="6">
+        <v>0</v>
+      </c>
+      <c r="F132" s="6">
+        <v>0</v>
+      </c>
+      <c r="G132" s="6">
+        <v>0</v>
+      </c>
+      <c r="H132" s="7">
+        <v>99615</v>
+      </c>
+      <c r="I132" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="J132" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="K132" s="6" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="133" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A133" s="6">
+        <v>16</v>
+      </c>
+      <c r="B133" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="C133" s="6">
+        <v>3</v>
+      </c>
+      <c r="D133" s="6">
+        <v>12</v>
+      </c>
+      <c r="E133" s="6">
+        <v>1</v>
+      </c>
+      <c r="F133" s="6">
+        <v>0</v>
+      </c>
+      <c r="G133" s="6">
+        <v>0</v>
+      </c>
+      <c r="H133" s="7">
+        <v>46806</v>
+      </c>
+      <c r="I133" s="7">
+        <v>1984</v>
+      </c>
+      <c r="J133" s="6">
+        <v>161</v>
+      </c>
+      <c r="K133" s="7">
+        <v>8688</v>
+      </c>
+    </row>
+    <row r="134" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A134" s="6">
+        <v>16</v>
+      </c>
+      <c r="B134" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="C134" s="6">
+        <v>3</v>
+      </c>
+      <c r="D134" s="6">
+        <v>12</v>
+      </c>
+      <c r="E134" s="6">
+        <v>0</v>
+      </c>
+      <c r="F134" s="6">
+        <v>0</v>
+      </c>
+      <c r="G134" s="6">
+        <v>0</v>
+      </c>
+      <c r="H134" s="7">
+        <v>48846</v>
+      </c>
+      <c r="I134" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="J134" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="K134" s="6" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="135" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A135" s="6">
+        <v>16</v>
+      </c>
+      <c r="B135" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="C135" s="6">
+        <v>3</v>
+      </c>
+      <c r="D135" s="6">
+        <v>12</v>
+      </c>
+      <c r="E135" s="6">
+        <v>0</v>
+      </c>
+      <c r="F135" s="6">
+        <v>0</v>
+      </c>
+      <c r="G135" s="6">
+        <v>0</v>
+      </c>
+      <c r="H135" s="7">
+        <v>47044</v>
+      </c>
+      <c r="I135" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="J135" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="K135" s="6" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="136" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A136" s="6">
+        <v>16</v>
+      </c>
+      <c r="B136" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="C136" s="6">
+        <v>3</v>
+      </c>
+      <c r="D136" s="6">
+        <v>12</v>
+      </c>
+      <c r="E136" s="6">
+        <v>0</v>
+      </c>
+      <c r="F136" s="6">
+        <v>0</v>
+      </c>
+      <c r="G136" s="6">
+        <v>0</v>
+      </c>
+      <c r="H136" s="7">
+        <v>44626</v>
+      </c>
+      <c r="I136" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="J136" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="K136" s="6" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="137" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A137" s="6">
+        <v>16</v>
+      </c>
+      <c r="B137" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="C137" s="6">
+        <v>6</v>
+      </c>
+      <c r="D137" s="6">
+        <v>24</v>
+      </c>
+      <c r="E137" s="6">
+        <v>0</v>
+      </c>
+      <c r="F137" s="6">
+        <v>0</v>
+      </c>
+      <c r="G137" s="6">
+        <v>0</v>
+      </c>
+      <c r="H137" s="7">
+        <v>85965</v>
+      </c>
+      <c r="I137" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="J137" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="K137" s="6" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="138" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A138" s="6">
+        <v>16</v>
+      </c>
+      <c r="B138" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="C138" s="6">
+        <v>5</v>
+      </c>
+      <c r="D138" s="6">
+        <v>20</v>
+      </c>
+      <c r="E138" s="6">
+        <v>0</v>
+      </c>
+      <c r="F138" s="6">
+        <v>0</v>
+      </c>
+      <c r="G138" s="6">
+        <v>0</v>
+      </c>
+      <c r="H138" s="7">
+        <v>69086</v>
+      </c>
+      <c r="I138" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="J138" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="K138" s="6" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="139" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A139" s="6">
+        <v>16</v>
+      </c>
+      <c r="B139" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="C139" s="6">
+        <v>32</v>
+      </c>
+      <c r="D139" s="6">
+        <v>128</v>
+      </c>
+      <c r="E139" s="6">
+        <v>1</v>
+      </c>
+      <c r="F139" s="6">
+        <v>0</v>
+      </c>
+      <c r="G139" s="6">
+        <v>0</v>
+      </c>
+      <c r="H139" s="7">
+        <v>493964</v>
+      </c>
+      <c r="I139" s="7">
+        <v>1984</v>
+      </c>
+      <c r="J139" s="6">
+        <v>161</v>
+      </c>
+      <c r="K139" s="7">
+        <v>8688</v>
       </c>
     </row>
   </sheetData>
@@ -5097,14 +5439,14 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DC5A6928-3806-4082-94AB-A52936AB7317}">
-  <dimension ref="A1:B16"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:B18"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="5.6640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="27.5546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="5.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="27.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
@@ -5112,7 +5454,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
@@ -5120,7 +5462,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2</v>
       </c>
@@ -5128,7 +5470,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>3</v>
       </c>
@@ -5136,7 +5478,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>4</v>
       </c>
@@ -5144,7 +5486,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>5</v>
       </c>
@@ -5152,7 +5494,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>6</v>
       </c>
@@ -5160,7 +5502,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>7</v>
       </c>
@@ -5168,7 +5510,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>8</v>
       </c>
@@ -5176,7 +5518,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>9</v>
       </c>
@@ -5184,7 +5526,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>10</v>
       </c>
@@ -5192,7 +5534,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>11</v>
       </c>
@@ -5200,7 +5542,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>12</v>
       </c>
@@ -5208,7 +5550,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>13</v>
       </c>
@@ -5216,7 +5558,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>14</v>
       </c>
@@ -5224,13 +5566,24 @@
         <v>36</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>15</v>
       </c>
       <c r="B16" t="s">
         <v>37</v>
       </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A17" s="6">
+        <v>16</v>
+      </c>
+      <c r="B17" s="5" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A18" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>